<commit_message>
data: update NA Bench Forecast — 2026-09-01 13:18
</commit_message>
<xml_diff>
--- a/NA Bench Forecast.xlsx
+++ b/NA Bench Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbondcrx/Desktop/BOB!/Bench Forecast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{46750368-C903-3C46-994B-88100D504DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D94E56-12DC-0349-8394-1A55BBBBE2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="600" windowWidth="27320" windowHeight="16080" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="180" yWindow="660" windowWidth="27320" windowHeight="16080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench Forecast" sheetId="1" r:id="rId1"/>
@@ -29,10 +29,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="212" r:id="rId8"/>
-    <pivotCache cacheId="217" r:id="rId9"/>
+    <pivotCache cacheId="19" r:id="rId8"/>
+    <pivotCache cacheId="22" r:id="rId9"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -50,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="172">
   <si>
     <t>Center</t>
   </si>
@@ -561,6 +560,12 @@
   <si>
     <t xml:space="preserve">  Wk 13</t>
   </si>
+  <si>
+    <t>3Q26 WK9</t>
+  </si>
+  <si>
+    <t>3Q26 WK8</t>
+  </si>
 </sst>
 </file>
 
@@ -569,7 +574,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1003,6 +1008,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
@@ -1022,38 +1031,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -1305,22 +1290,22 @@
                   <c:v>7.6999503229011432E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.9483358171882762E-2</c:v>
+                  <c:v>7.1038251366120214E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.9980129160457034E-2</c:v>
+                  <c:v>7.1535022354694486E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.10084451068057626</c:v>
+                  <c:v>8.1470442126179834E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.10680576254346746</c:v>
+                  <c:v>8.3954297069051165E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.10630899155489319</c:v>
+                  <c:v>8.5444610034773966E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.10481867858917039</c:v>
+                  <c:v>8.5941381023348237E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1919,9 +1904,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Historic Bench Data'!$Q$24:$Q$108</c:f>
+              <c:f>'Historic Bench Data'!$Q$24:$Q$110</c:f>
               <c:strCache>
-                <c:ptCount val="84"/>
+                <c:ptCount val="86"/>
                 <c:pt idx="0">
                   <c:v>1Q WK 01</c:v>
                 </c:pt>
@@ -2173,16 +2158,22 @@
                 </c:pt>
                 <c:pt idx="83">
                   <c:v>3Q26 WK7</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>3Q26 WK8</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>3Q26 WK9</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Historic Bench Data'!$R$24:$R$108</c:f>
+              <c:f>'Historic Bench Data'!$R$24:$R$110</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="84"/>
+                <c:ptCount val="86"/>
                 <c:pt idx="0">
                   <c:v>268</c:v>
                 </c:pt>
@@ -2434,6 +2425,12 @@
                 </c:pt>
                 <c:pt idx="83">
                   <c:v>155</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>149</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>145</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11592,6 +11589,111 @@
           </c:spPr>
         </c:marker>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="142"/>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr/>
+              </a:pPr>
+              <a:endParaRPr lang="en-CR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="143"/>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr/>
+              </a:pPr>
+              <a:endParaRPr lang="en-CR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="144"/>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr/>
+              </a:pPr>
+              <a:endParaRPr lang="en-CR"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="ctr"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout>
@@ -11630,6 +11732,18 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:endParaRPr lang="en-CR"/>
+              </a:p>
+            </c:txPr>
             <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
@@ -11768,6 +11882,18 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:endParaRPr lang="en-CR"/>
+              </a:p>
+            </c:txPr>
             <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
@@ -11906,6 +12032,18 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:txPr>
+              <a:bodyPr wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:endParaRPr lang="en-CR"/>
+              </a:p>
+            </c:txPr>
             <c:dLblPos val="ctr"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
@@ -12245,16 +12383,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3973</xdr:colOff>
-      <xdr:row>107</xdr:row>
-      <xdr:rowOff>132690</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>103</xdr:row>
+      <xdr:rowOff>104778</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>100794</xdr:colOff>
-      <xdr:row>132</xdr:row>
-      <xdr:rowOff>100793</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>515503</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>72882</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -12568,13 +12706,74 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46252.573241550926" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="84" xr:uid="{00000000-000A-0000-FFFF-FFFF97000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46255.600433680556" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{00000000-000A-0000-FFFF-FFFF9B000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="N2:O86" sheet="Historic Bench Data"/>
+    <worksheetSource ref="A30:N33" sheet="Q3 2025"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="Total Bench" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Q3 26 Forecast"/>
+        <s v="Q3 25 bench"/>
+        <s v="Q3 Original Forecast"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Wk 01" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="159" maxValue="170"/>
+    </cacheField>
+    <cacheField name="Wk 02" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="148" maxValue="166"/>
+    </cacheField>
+    <cacheField name="Wk 03" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="133" maxValue="158"/>
+    </cacheField>
+    <cacheField name="Wk 04" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="138" maxValue="156"/>
+    </cacheField>
+    <cacheField name="Wk 05" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="121" maxValue="152"/>
+    </cacheField>
+    <cacheField name="Wk 06" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="136" maxValue="165"/>
+    </cacheField>
+    <cacheField name="Wk 07" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="119" maxValue="175"/>
+    </cacheField>
+    <cacheField name="Wk 08" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="114" maxValue="176"/>
+    </cacheField>
+    <cacheField name="Wk 09" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="171"/>
+    </cacheField>
+    <cacheField name="Wk 10" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="112" maxValue="203"/>
+    </cacheField>
+    <cacheField name="Wk 11" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="215"/>
+    </cacheField>
+    <cacheField name="Wk 12" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="95" maxValue="214"/>
+    </cacheField>
+    <cacheField name="Wk 13" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="211"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46266.442498611112" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="86" xr:uid="{C61BEA90-B2FA-4A48-9A9E-52FD3131D3A2}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="N2:O88" sheet="Historic Bench Data"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Wk" numFmtId="0">
-      <sharedItems count="84">
+      <sharedItems count="86">
         <s v="1Q WK 01"/>
         <s v="1Q WK 02"/>
         <s v="1Q WK 03"/>
@@ -12659,6 +12858,8 @@
         <s v="3Q26 WK5"/>
         <s v="3Q26 WK6"/>
         <s v="3Q26 WK7"/>
+        <s v="3Q26 WK8"/>
+        <s v="3Q26 WK9"/>
       </sharedItems>
     </cacheField>
     <cacheField name="NA CIC" numFmtId="0">
@@ -12673,69 +12874,61 @@
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46255.600433680556" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{00000000-000A-0000-FFFF-FFFF9B000000}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A30:N33" sheet="Q3 2025"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="Total Bench" numFmtId="0">
-      <sharedItems count="3">
-        <s v="Q3 26 Forecast"/>
-        <s v="Q3 25 bench"/>
-        <s v="Q3 Original Forecast"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Wk 01" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="159" maxValue="170"/>
-    </cacheField>
-    <cacheField name="Wk 02" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="148" maxValue="166"/>
-    </cacheField>
-    <cacheField name="Wk 03" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="133" maxValue="158"/>
-    </cacheField>
-    <cacheField name="Wk 04" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="138" maxValue="156"/>
-    </cacheField>
-    <cacheField name="Wk 05" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="121" maxValue="152"/>
-    </cacheField>
-    <cacheField name="Wk 06" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="136" maxValue="165"/>
-    </cacheField>
-    <cacheField name="Wk 07" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="119" maxValue="175"/>
-    </cacheField>
-    <cacheField name="Wk 08" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="114" maxValue="176"/>
-    </cacheField>
-    <cacheField name="Wk 09" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="171"/>
-    </cacheField>
-    <cacheField name="Wk 10" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="112" maxValue="203"/>
-    </cacheField>
-    <cacheField name="Wk 11" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="215"/>
-    </cacheField>
-    <cacheField name="Wk 12" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="95" maxValue="214"/>
-    </cacheField>
-    <cacheField name="Wk 13" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="211"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
+  <r>
+    <x v="0"/>
+    <n v="170"/>
+    <n v="166"/>
+    <n v="158"/>
+    <n v="138"/>
+    <n v="130"/>
+    <n v="147"/>
+    <n v="155"/>
+    <n v="160"/>
+    <n v="161"/>
+    <n v="203"/>
+    <n v="215"/>
+    <n v="214"/>
+    <n v="211"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="159"/>
+    <n v="148"/>
+    <n v="133"/>
+    <n v="138"/>
+    <n v="121"/>
+    <n v="136"/>
+    <n v="119"/>
+    <n v="114"/>
+    <n v="104"/>
+    <n v="112"/>
+    <n v="98"/>
+    <n v="95"/>
+    <n v="89"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="159"/>
+    <n v="161"/>
+    <n v="154"/>
+    <n v="156"/>
+    <n v="152"/>
+    <n v="165"/>
+    <n v="175"/>
+    <n v="176"/>
+    <n v="171"/>
+    <n v="196"/>
+    <n v="192"/>
+    <n v="191"/>
+    <n v="187"/>
+  </r>
+</pivotCacheRecords>
 </file>
 
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84">
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="86">
   <r>
     <x v="0"/>
     <n v="268"/>
@@ -13072,68 +13265,23 @@
     <x v="83"/>
     <n v="155"/>
   </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
   <r>
-    <x v="0"/>
-    <n v="170"/>
-    <n v="166"/>
-    <n v="158"/>
-    <n v="138"/>
-    <n v="130"/>
-    <n v="147"/>
-    <n v="155"/>
-    <n v="160"/>
-    <n v="161"/>
-    <n v="203"/>
-    <n v="215"/>
-    <n v="214"/>
-    <n v="211"/>
+    <x v="84"/>
+    <n v="149"/>
   </r>
   <r>
-    <x v="1"/>
-    <n v="159"/>
-    <n v="148"/>
-    <n v="133"/>
-    <n v="138"/>
-    <n v="121"/>
-    <n v="136"/>
-    <n v="119"/>
-    <n v="114"/>
-    <n v="104"/>
-    <n v="112"/>
-    <n v="98"/>
-    <n v="95"/>
-    <n v="89"/>
-  </r>
-  <r>
-    <x v="2"/>
-    <n v="159"/>
-    <n v="161"/>
-    <n v="154"/>
-    <n v="156"/>
-    <n v="152"/>
-    <n v="165"/>
-    <n v="175"/>
-    <n v="176"/>
-    <n v="171"/>
-    <n v="196"/>
-    <n v="192"/>
-    <n v="191"/>
-    <n v="187"/>
+    <x v="85"/>
+    <n v="145"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable12" cacheId="212" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
-  <location ref="Q23:R108" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C7F007FE-B437-4141-95D7-2E6144C3BF9C}" name="PivotTable12" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+  <location ref="Q23:R110" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
-      <items count="85">
+      <items count="87">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -13218,6 +13366,8 @@
         <item x="81"/>
         <item x="82"/>
         <item x="83"/>
+        <item x="84"/>
+        <item x="85"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -13226,7 +13376,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="85">
+  <rowItems count="87">
     <i>
       <x/>
     </i>
@@ -13479,6 +13629,12 @@
     <i>
       <x v="83"/>
     </i>
+    <i>
+      <x v="84"/>
+    </i>
+    <i>
+      <x v="85"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
@@ -13579,7 +13735,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable2" cacheId="217" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="44">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable2" cacheId="19" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="44">
   <location ref="A36:E50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisCol" showAll="0">
@@ -13681,7 +13837,7 @@
     <dataField name="  Wk 13" fld="13" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="11">
+    <format dxfId="5">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="13">
@@ -13702,27 +13858,27 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="4">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="3">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="2">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
-  <chartFormats count="82">
+  <chartFormats count="85">
     <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -14668,6 +14824,42 @@
         </references>
       </pivotArea>
     </chartFormat>
+    <chartFormat chart="43" format="142" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="43" format="143" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="43" format="144" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -14996,7 +15188,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" outlineLevelCol="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" outlineLevelCol="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
     <col min="2" max="2" width="8" style="1" customWidth="1" outlineLevel="1"/>
@@ -15005,7 +15197,7 @@
     <col min="5" max="14" width="10.5" style="1" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -15049,7 +15241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>14</v>
       </c>
@@ -15074,11 +15266,11 @@
       <c r="H2" s="12">
         <v>43</v>
       </c>
-      <c r="I2" s="8">
-        <v>38</v>
-      </c>
-      <c r="J2" s="8">
-        <v>36</v>
+      <c r="I2" s="12">
+        <v>37</v>
+      </c>
+      <c r="J2" s="12">
+        <v>37</v>
       </c>
       <c r="K2" s="8">
         <v>49</v>
@@ -15093,7 +15285,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>15</v>
       </c>
@@ -15118,10 +15310,10 @@
       <c r="H3" s="12">
         <v>2</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="12">
         <v>3</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="12">
         <v>4</v>
       </c>
       <c r="K3" s="11">
@@ -15137,7 +15329,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
@@ -15162,11 +15354,11 @@
       <c r="H4" s="12">
         <v>41</v>
       </c>
-      <c r="I4" s="8">
-        <v>28</v>
-      </c>
-      <c r="J4" s="8">
-        <v>29</v>
+      <c r="I4" s="12">
+        <v>36</v>
+      </c>
+      <c r="J4" s="12">
+        <v>37</v>
       </c>
       <c r="K4" s="8">
         <v>33</v>
@@ -15181,7 +15373,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>17</v>
       </c>
@@ -15206,26 +15398,26 @@
       <c r="H5" s="12">
         <v>23</v>
       </c>
-      <c r="I5" s="11">
-        <v>49</v>
-      </c>
-      <c r="J5" s="11">
-        <v>47</v>
+      <c r="I5" s="12">
+        <v>22</v>
+      </c>
+      <c r="J5" s="12">
+        <v>24</v>
       </c>
       <c r="K5" s="11">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="L5" s="11">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="M5" s="11">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="N5" s="11">
-        <v>64</v>
+        <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>18</v>
       </c>
@@ -15250,11 +15442,11 @@
       <c r="H6" s="12">
         <v>15</v>
       </c>
-      <c r="I6" s="8">
-        <v>10</v>
-      </c>
-      <c r="J6" s="8">
-        <v>10</v>
+      <c r="I6" s="12">
+        <v>14</v>
+      </c>
+      <c r="J6" s="12">
+        <v>13</v>
       </c>
       <c r="K6" s="8">
         <v>13</v>
@@ -15269,7 +15461,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>19</v>
       </c>
@@ -15294,11 +15486,11 @@
       <c r="H7" s="12">
         <v>12</v>
       </c>
-      <c r="I7" s="11">
-        <v>13</v>
-      </c>
-      <c r="J7" s="11">
-        <v>13</v>
+      <c r="I7" s="12">
+        <v>12</v>
+      </c>
+      <c r="J7" s="12">
+        <v>10</v>
       </c>
       <c r="K7" s="11">
         <v>14</v>
@@ -15313,7 +15505,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>20</v>
       </c>
@@ -15338,26 +15530,26 @@
       <c r="H8" s="12">
         <v>19</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="12">
         <v>19</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="12">
+        <v>19</v>
+      </c>
+      <c r="K8" s="8">
         <v>22</v>
       </c>
-      <c r="K8" s="8">
-        <v>31</v>
-      </c>
       <c r="L8" s="8">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="M8" s="8">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="N8" s="8">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -15391,30 +15583,30 @@
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="J9" s="6">
         <f t="shared" si="0"/>
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="K9" s="6">
         <f t="shared" si="0"/>
-        <v>203</v>
+        <v>164</v>
       </c>
       <c r="L9" s="6">
         <f t="shared" si="0"/>
-        <v>215</v>
+        <v>169</v>
       </c>
       <c r="M9" s="6">
         <f t="shared" si="0"/>
-        <v>214</v>
+        <v>172</v>
       </c>
       <c r="N9" s="6">
         <f t="shared" si="0"/>
-        <v>211</v>
+        <v>173</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
@@ -15448,30 +15640,30 @@
       </c>
       <c r="I10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9483358171882762E-2</v>
+        <v>7.1038251366120214E-2</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9980129160457034E-2</v>
+        <v>7.1535022354694486E-2</v>
       </c>
       <c r="K10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10084451068057626</v>
+        <v>8.1470442126179834E-2</v>
       </c>
       <c r="L10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10680576254346746</v>
+        <v>8.3954297069051165E-2</v>
       </c>
       <c r="M10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10630899155489319</v>
+        <v>8.5444610034773966E-2</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10481867858917039</v>
+        <v>8.5941381023348237E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>23</v>
       </c>
@@ -15480,21 +15672,14 @@
       </c>
       <c r="C11" s="10"/>
     </row>
-    <row r="16" spans="1:14">
-      <c r="N16">
-        <v>136</v>
-      </c>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="N16"/>
     </row>
-    <row r="17" spans="14:14">
-      <c r="N17">
-        <v>180</v>
-      </c>
+    <row r="17" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N17"/>
     </row>
-    <row r="18" spans="14:14">
-      <c r="N18">
-        <f>+N17-N16</f>
-        <v>44</v>
-      </c>
+    <row r="18" spans="14:14" x14ac:dyDescent="0.2">
+      <c r="N18"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -15505,8 +15690,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R108"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16"/>
+  <dimension ref="A1:R110"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -15518,11 +15703,10 @@
     <col min="9" max="9" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="18" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32" customHeight="1">
+    <row r="1" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>24</v>
       </c>
@@ -15560,7 +15744,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="14">
         <v>2025</v>
       </c>
@@ -15606,7 +15790,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="14">
         <v>2025</v>
       </c>
@@ -15652,7 +15836,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="14">
         <v>2025</v>
       </c>
@@ -15698,7 +15882,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="14">
         <v>2025</v>
       </c>
@@ -15744,7 +15928,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="14">
         <v>2025</v>
       </c>
@@ -15790,7 +15974,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="14">
         <v>2025</v>
       </c>
@@ -15836,7 +16020,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="14">
         <v>2025</v>
       </c>
@@ -15882,7 +16066,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="14">
         <v>2025</v>
       </c>
@@ -15928,7 +16112,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="14">
         <v>2025</v>
       </c>
@@ -15974,7 +16158,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="14">
         <v>2025</v>
       </c>
@@ -16020,7 +16204,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="14">
         <v>2025</v>
       </c>
@@ -16066,7 +16250,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="14">
         <v>2025</v>
       </c>
@@ -16112,7 +16296,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="14">
         <v>2025</v>
       </c>
@@ -16158,7 +16342,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="14">
         <v>2025</v>
       </c>
@@ -16204,7 +16388,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="14">
         <v>2025</v>
       </c>
@@ -16250,7 +16434,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="14">
         <v>2025</v>
       </c>
@@ -16296,7 +16480,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="18" spans="1:18">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="14">
         <v>2025</v>
       </c>
@@ -16342,7 +16526,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:18">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" s="14">
         <v>2025</v>
       </c>
@@ -16388,7 +16572,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="20" spans="1:18">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" s="14">
         <v>2025</v>
       </c>
@@ -16434,7 +16618,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="21" spans="1:18">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" s="14">
         <v>2025</v>
       </c>
@@ -16480,7 +16664,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="22" spans="1:18">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="14">
         <v>2025</v>
       </c>
@@ -16526,7 +16710,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="23" spans="1:18">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" s="14">
         <v>2025</v>
       </c>
@@ -16578,7 +16762,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" s="14">
         <v>2025</v>
       </c>
@@ -16626,11 +16810,11 @@
       <c r="Q24" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="R24">
+      <c r="R24" s="50">
         <v>268</v>
       </c>
     </row>
-    <row r="25" spans="1:18">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="14">
         <v>2025</v>
       </c>
@@ -16678,11 +16862,11 @@
       <c r="Q25" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="R25">
+      <c r="R25" s="50">
         <v>290</v>
       </c>
     </row>
-    <row r="26" spans="1:18">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="14">
         <v>2025</v>
       </c>
@@ -16730,11 +16914,11 @@
       <c r="Q26" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="R26">
+      <c r="R26" s="50">
         <v>227</v>
       </c>
     </row>
-    <row r="27" spans="1:18">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="14">
         <v>2025</v>
       </c>
@@ -16782,11 +16966,11 @@
       <c r="Q27" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="R27">
+      <c r="R27" s="50">
         <v>228</v>
       </c>
     </row>
-    <row r="28" spans="1:18">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="14">
         <v>2025</v>
       </c>
@@ -16834,11 +17018,11 @@
       <c r="Q28" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="R28">
+      <c r="R28" s="50">
         <v>214</v>
       </c>
     </row>
-    <row r="29" spans="1:18">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="14">
         <v>2025</v>
       </c>
@@ -16886,11 +17070,11 @@
       <c r="Q29" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="R29">
+      <c r="R29" s="50">
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:18">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" s="14">
         <v>2025</v>
       </c>
@@ -16938,11 +17122,11 @@
       <c r="Q30" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="R30">
+      <c r="R30" s="50">
         <v>207</v>
       </c>
     </row>
-    <row r="31" spans="1:18">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" s="14">
         <v>2025</v>
       </c>
@@ -16990,11 +17174,11 @@
       <c r="Q31" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="R31">
+      <c r="R31" s="50">
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:18">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" s="14">
         <v>2025</v>
       </c>
@@ -17042,11 +17226,11 @@
       <c r="Q32" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="R32">
+      <c r="R32" s="50">
         <v>189</v>
       </c>
     </row>
-    <row r="33" spans="1:18">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="14">
         <v>2025</v>
       </c>
@@ -17093,11 +17277,11 @@
       <c r="Q33" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="R33">
+      <c r="R33" s="50">
         <v>180</v>
       </c>
     </row>
-    <row r="34" spans="1:18">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" s="14">
         <v>2025</v>
       </c>
@@ -17144,11 +17328,11 @@
       <c r="Q34" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="R34">
+      <c r="R34" s="50">
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:18">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" s="14">
         <v>2025</v>
       </c>
@@ -17196,11 +17380,11 @@
       <c r="Q35" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="R35">
+      <c r="R35" s="50">
         <v>154</v>
       </c>
     </row>
-    <row r="36" spans="1:18">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36" s="14">
         <v>2025</v>
       </c>
@@ -17247,11 +17431,11 @@
       <c r="Q36" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="R36">
+      <c r="R36" s="50">
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:18">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37" s="14">
         <v>2025</v>
       </c>
@@ -17298,11 +17482,11 @@
       <c r="Q37" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="R37">
+      <c r="R37" s="50">
         <v>169</v>
       </c>
     </row>
-    <row r="38" spans="1:18">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" s="14">
         <v>2025</v>
       </c>
@@ -17349,11 +17533,11 @@
       <c r="Q38" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="R38">
+      <c r="R38" s="50">
         <v>142</v>
       </c>
     </row>
-    <row r="39" spans="1:18">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="14">
         <v>2025</v>
       </c>
@@ -17400,11 +17584,11 @@
       <c r="Q39" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="R39">
+      <c r="R39" s="50">
         <v>169</v>
       </c>
     </row>
-    <row r="40" spans="1:18">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40" s="14">
         <v>2025</v>
       </c>
@@ -17451,11 +17635,11 @@
       <c r="Q40" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="R40">
+      <c r="R40" s="50">
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:18">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41" s="14">
         <v>2025</v>
       </c>
@@ -17503,11 +17687,11 @@
       <c r="Q41" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R41">
+      <c r="R41" s="50">
         <v>164</v>
       </c>
     </row>
-    <row r="42" spans="1:18">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A42" s="14">
         <v>2025</v>
       </c>
@@ -17555,11 +17739,11 @@
       <c r="Q42" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="R42">
+      <c r="R42" s="50">
         <v>136</v>
       </c>
     </row>
-    <row r="43" spans="1:18">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A43" s="14">
         <v>2025</v>
       </c>
@@ -17607,11 +17791,11 @@
       <c r="Q43" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="R43">
+      <c r="R43" s="50">
         <v>147</v>
       </c>
     </row>
-    <row r="44" spans="1:18">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A44" s="14">
         <v>2025</v>
       </c>
@@ -17659,11 +17843,11 @@
       <c r="Q44" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="R44">
+      <c r="R44" s="50">
         <v>146</v>
       </c>
     </row>
-    <row r="45" spans="1:18">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45" s="14">
         <v>2025</v>
       </c>
@@ -17711,11 +17895,11 @@
       <c r="Q45" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="R45">
+      <c r="R45" s="50">
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:18">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46" s="14">
         <v>2025</v>
       </c>
@@ -17763,11 +17947,11 @@
       <c r="Q46" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="R46">
+      <c r="R46" s="50">
         <v>161</v>
       </c>
     </row>
-    <row r="47" spans="1:18">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47" s="14">
         <v>2025</v>
       </c>
@@ -17815,11 +17999,11 @@
       <c r="Q47" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="R47">
+      <c r="R47" s="50">
         <v>159</v>
       </c>
     </row>
-    <row r="48" spans="1:18">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A48" s="14">
         <v>2025</v>
       </c>
@@ -17867,11 +18051,11 @@
       <c r="Q48" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="R48">
+      <c r="R48" s="50">
         <v>133</v>
       </c>
     </row>
-    <row r="49" spans="1:18">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A49" s="14">
         <v>2025</v>
       </c>
@@ -17919,11 +18103,11 @@
       <c r="Q49" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="R49">
+      <c r="R49" s="50">
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:18">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A50" s="14">
         <v>2025</v>
       </c>
@@ -17971,11 +18155,11 @@
       <c r="Q50" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="R50">
+      <c r="R50" s="50">
         <v>181</v>
       </c>
     </row>
-    <row r="51" spans="1:18">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51" s="14">
         <v>2025</v>
       </c>
@@ -18023,11 +18207,11 @@
       <c r="Q51" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="R51">
+      <c r="R51" s="50">
         <v>177</v>
       </c>
     </row>
-    <row r="52" spans="1:18">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52" s="14">
         <v>2025</v>
       </c>
@@ -18075,11 +18259,11 @@
       <c r="Q52" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="R52">
+      <c r="R52" s="50">
         <v>165</v>
       </c>
     </row>
-    <row r="53" spans="1:18">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53" s="14">
         <v>2025</v>
       </c>
@@ -18127,11 +18311,11 @@
       <c r="Q53" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="R53">
+      <c r="R53" s="50">
         <v>168</v>
       </c>
     </row>
-    <row r="54" spans="1:18">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A54" s="14">
         <v>2026</v>
       </c>
@@ -18179,11 +18363,11 @@
       <c r="Q54" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="R54">
+      <c r="R54" s="50">
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:18">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A55" s="14">
         <v>2026</v>
       </c>
@@ -18231,11 +18415,11 @@
       <c r="Q55" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="R55">
+      <c r="R55" s="50">
         <v>156</v>
       </c>
     </row>
-    <row r="56" spans="1:18">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A56" s="14">
         <v>2026</v>
       </c>
@@ -18283,11 +18467,11 @@
       <c r="Q56" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="R56">
+      <c r="R56" s="50">
         <v>158</v>
       </c>
     </row>
-    <row r="57" spans="1:18">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A57" s="14">
         <v>2026</v>
       </c>
@@ -18335,11 +18519,11 @@
       <c r="Q57" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="R57">
+      <c r="R57" s="50">
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:18">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A58" s="14">
         <v>2026</v>
       </c>
@@ -18387,11 +18571,11 @@
       <c r="Q58" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="R58">
+      <c r="R58" s="50">
         <v>128</v>
       </c>
     </row>
-    <row r="59" spans="1:18">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A59" s="14">
         <v>2026</v>
       </c>
@@ -18439,11 +18623,11 @@
       <c r="Q59" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="R59">
+      <c r="R59" s="50">
         <v>134</v>
       </c>
     </row>
-    <row r="60" spans="1:18">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A60" s="14">
         <v>2026</v>
       </c>
@@ -18491,11 +18675,11 @@
       <c r="Q60" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="R60">
+      <c r="R60" s="50">
         <v>123</v>
       </c>
     </row>
-    <row r="61" spans="1:18">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A61" s="14">
         <v>2026</v>
       </c>
@@ -18543,11 +18727,11 @@
       <c r="Q61" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="R61">
+      <c r="R61" s="50">
         <v>123</v>
       </c>
     </row>
-    <row r="62" spans="1:18">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A62" s="14">
         <v>2026</v>
       </c>
@@ -18595,11 +18779,11 @@
       <c r="Q62" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="R62">
+      <c r="R62" s="50">
         <v>112</v>
       </c>
     </row>
-    <row r="63" spans="1:18">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A63" s="14">
         <v>2026</v>
       </c>
@@ -18647,11 +18831,11 @@
       <c r="Q63" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="R63">
+      <c r="R63" s="50">
         <v>119</v>
       </c>
     </row>
-    <row r="64" spans="1:18">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A64" s="14">
         <v>2026</v>
       </c>
@@ -18699,11 +18883,11 @@
       <c r="Q64" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="R64">
+      <c r="R64" s="50">
         <v>107</v>
       </c>
     </row>
-    <row r="65" spans="1:18">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A65" s="14">
         <v>2026</v>
       </c>
@@ -18751,11 +18935,11 @@
       <c r="Q65" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="R65">
+      <c r="R65" s="50">
         <v>110</v>
       </c>
     </row>
-    <row r="66" spans="1:18">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A66" s="14">
         <v>2026</v>
       </c>
@@ -18790,7 +18974,7 @@
         <v>121</v>
       </c>
       <c r="L66" t="str">
-        <f t="shared" ref="L66:L85" si="4">+B66&amp;" "&amp;C66</f>
+        <f t="shared" ref="L66:L88" si="4">+B66&amp;" "&amp;C66</f>
         <v>2Q WK 01</v>
       </c>
       <c r="N66" t="s">
@@ -18802,11 +18986,11 @@
       <c r="Q66" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="R66">
+      <c r="R66" s="50">
         <v>137</v>
       </c>
     </row>
-    <row r="67" spans="1:18">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A67" s="14">
         <v>2026</v>
       </c>
@@ -18853,11 +19037,11 @@
       <c r="Q67" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="R67">
+      <c r="R67" s="50">
         <v>124</v>
       </c>
     </row>
-    <row r="68" spans="1:18">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A68" s="14">
         <v>2026</v>
       </c>
@@ -18904,11 +19088,11 @@
       <c r="Q68" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="R68">
+      <c r="R68" s="50">
         <v>127</v>
       </c>
     </row>
-    <row r="69" spans="1:18">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A69" s="14">
         <v>2026</v>
       </c>
@@ -18955,11 +19139,11 @@
       <c r="Q69" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="R69">
+      <c r="R69" s="50">
         <v>101</v>
       </c>
     </row>
-    <row r="70" spans="1:18">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A70" s="14">
         <v>2026</v>
       </c>
@@ -19007,11 +19191,11 @@
       <c r="Q70" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="R70">
+      <c r="R70" s="50">
         <v>116</v>
       </c>
     </row>
-    <row r="71" spans="1:18">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A71" s="14">
         <v>2026</v>
       </c>
@@ -19066,11 +19250,11 @@
       <c r="Q71" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="R71">
+      <c r="R71" s="50">
         <v>124</v>
       </c>
     </row>
-    <row r="72" spans="1:18">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A72" s="14">
         <v>2026</v>
       </c>
@@ -19118,11 +19302,11 @@
       <c r="Q72" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="R72">
+      <c r="R72" s="50">
         <v>134</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="17" customHeight="1" thickBot="1">
+    <row r="73" spans="1:18" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="14">
         <v>2026</v>
       </c>
@@ -19177,11 +19361,11 @@
       <c r="Q73" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="R73">
+      <c r="R73" s="50">
         <v>113</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="18" customHeight="1" thickTop="1" thickBot="1">
+    <row r="74" spans="1:18" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="14">
         <v>2026</v>
       </c>
@@ -19229,11 +19413,11 @@
       <c r="Q74" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="R74">
+      <c r="R74" s="50">
         <v>118</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="18" customHeight="1" thickTop="1" thickBot="1">
+    <row r="75" spans="1:18" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="14">
         <v>2026</v>
       </c>
@@ -19288,11 +19472,11 @@
       <c r="Q75" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="R75">
+      <c r="R75" s="50">
         <v>127</v>
       </c>
     </row>
-    <row r="76" spans="1:18">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A76" s="14">
         <v>2026</v>
       </c>
@@ -19340,11 +19524,11 @@
       <c r="Q76" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="R76">
+      <c r="R76" s="50">
         <v>231</v>
       </c>
     </row>
-    <row r="77" spans="1:18">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A77" s="14">
         <v>2026</v>
       </c>
@@ -19399,11 +19583,11 @@
       <c r="Q77" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="R77">
+      <c r="R77" s="50">
         <v>201</v>
       </c>
     </row>
-    <row r="78" spans="1:18">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A78" s="14">
         <v>2026</v>
       </c>
@@ -19450,11 +19634,11 @@
       <c r="Q78" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="R78">
+      <c r="R78" s="50">
         <v>180</v>
       </c>
     </row>
-    <row r="79" spans="1:18">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A79" s="14">
         <v>2026</v>
       </c>
@@ -19486,7 +19670,7 @@
         <v>18</v>
       </c>
       <c r="K79" s="15">
-        <f t="shared" ref="K79:K85" si="6">SUM(D79:J79)</f>
+        <f t="shared" ref="K79:K87" si="6">SUM(D79:J79)</f>
         <v>176</v>
       </c>
       <c r="L79" t="str">
@@ -19502,11 +19686,11 @@
       <c r="Q79" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="R79">
+      <c r="R79" s="50">
         <v>171</v>
       </c>
     </row>
-    <row r="80" spans="1:18">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A80" s="14">
         <v>2026</v>
       </c>
@@ -19554,11 +19738,11 @@
       <c r="Q80" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="R80">
+      <c r="R80" s="50">
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:18">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A81" s="14">
         <v>2026</v>
       </c>
@@ -19606,11 +19790,11 @@
       <c r="Q81" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="R81">
+      <c r="R81" s="50">
         <v>143</v>
       </c>
     </row>
-    <row r="82" spans="1:18">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A82" s="14">
         <v>2026</v>
       </c>
@@ -19658,11 +19842,11 @@
       <c r="Q82" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="R82">
+      <c r="R82" s="50">
         <v>114</v>
       </c>
     </row>
-    <row r="83" spans="1:18">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A83" s="14">
         <v>2026</v>
       </c>
@@ -19710,11 +19894,11 @@
       <c r="Q83" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="R83">
+      <c r="R83" s="50">
         <v>110</v>
       </c>
     </row>
-    <row r="84" spans="1:18">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A84" s="14">
         <v>2026</v>
       </c>
@@ -19762,11 +19946,11 @@
       <c r="Q84" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="R84">
+      <c r="R84" s="50">
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:18">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A85" s="14">
         <v>2026</v>
       </c>
@@ -19814,11 +19998,49 @@
       <c r="Q85" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="R85">
+      <c r="R85" s="50">
         <v>101</v>
       </c>
     </row>
-    <row r="86" spans="1:18">
+    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A86" s="14">
+        <v>2026</v>
+      </c>
+      <c r="B86" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D86" s="16">
+        <v>43</v>
+      </c>
+      <c r="E86" s="16">
+        <v>14</v>
+      </c>
+      <c r="F86" s="16">
+        <v>12</v>
+      </c>
+      <c r="G86" s="16">
+        <v>3</v>
+      </c>
+      <c r="H86" s="16">
+        <v>22</v>
+      </c>
+      <c r="I86" s="16">
+        <v>19</v>
+      </c>
+      <c r="J86" s="16">
+        <v>36</v>
+      </c>
+      <c r="K86" s="15">
+        <f t="shared" si="6"/>
+        <v>149</v>
+      </c>
+      <c r="L86" t="str">
+        <f t="shared" si="4"/>
+        <v>3Q Wk 08</v>
+      </c>
       <c r="N86" t="s">
         <v>132</v>
       </c>
@@ -19828,184 +20050,254 @@
       <c r="Q86" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="R86">
+      <c r="R86" s="50">
         <v>78</v>
       </c>
     </row>
-    <row r="87" spans="1:18">
+    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A87" s="14">
+        <v>2026</v>
+      </c>
+      <c r="B87" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C87" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D87" s="16">
+        <v>37</v>
+      </c>
+      <c r="E87" s="16">
+        <v>13</v>
+      </c>
+      <c r="F87" s="16">
+        <v>10</v>
+      </c>
+      <c r="G87" s="16">
+        <v>4</v>
+      </c>
+      <c r="H87" s="16">
+        <v>24</v>
+      </c>
+      <c r="I87" s="16">
+        <v>20</v>
+      </c>
+      <c r="J87" s="16">
+        <v>37</v>
+      </c>
+      <c r="K87" s="15">
+        <f t="shared" si="6"/>
+        <v>145</v>
+      </c>
+      <c r="L87" t="str">
+        <f t="shared" si="4"/>
+        <v>3Q Wk 09</v>
+      </c>
+      <c r="N87" t="s">
+        <v>171</v>
+      </c>
+      <c r="O87">
+        <v>149</v>
+      </c>
       <c r="Q87" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="R87">
+      <c r="R87" s="50">
         <v>73</v>
       </c>
     </row>
-    <row r="88" spans="1:18">
+    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="L88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="N88" t="s">
+        <v>170</v>
+      </c>
+      <c r="O88">
+        <v>145</v>
+      </c>
       <c r="Q88" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="R88">
+      <c r="R88" s="50">
         <v>121</v>
       </c>
     </row>
-    <row r="89" spans="1:18">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q89" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="R89">
+      <c r="R89" s="50">
         <v>117</v>
       </c>
     </row>
-    <row r="90" spans="1:18">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q90" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="R90">
+      <c r="R90" s="50">
         <v>114</v>
       </c>
     </row>
-    <row r="91" spans="1:18">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q91" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="R91">
+      <c r="R91" s="50">
         <v>114</v>
       </c>
     </row>
-    <row r="92" spans="1:18">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q92" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="R92">
+      <c r="R92" s="50">
         <v>114</v>
       </c>
     </row>
-    <row r="93" spans="1:18">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q93" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="R93">
+      <c r="R93" s="50">
         <v>137</v>
       </c>
     </row>
-    <row r="94" spans="1:18">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q94" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="R94">
+      <c r="R94" s="50">
         <v>126</v>
       </c>
     </row>
-    <row r="95" spans="1:18">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q95" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="R95">
+      <c r="R95" s="50">
         <v>151</v>
       </c>
     </row>
-    <row r="96" spans="1:18">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
       <c r="Q96" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="R96">
+      <c r="R96" s="50">
         <v>125</v>
       </c>
     </row>
-    <row r="97" spans="17:18">
+    <row r="97" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q97" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="R97">
+      <c r="R97" s="50">
         <v>116</v>
       </c>
     </row>
-    <row r="98" spans="17:18">
+    <row r="98" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q98" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="R98">
+      <c r="R98" s="50">
         <v>145</v>
       </c>
     </row>
-    <row r="99" spans="17:18">
+    <row r="99" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q99" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="R99">
+      <c r="R99" s="50">
         <v>148</v>
       </c>
     </row>
-    <row r="100" spans="17:18">
+    <row r="100" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q100" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="R100">
+      <c r="R100" s="50">
         <v>152</v>
       </c>
     </row>
-    <row r="101" spans="17:18">
+    <row r="101" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q101" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="R101">
+      <c r="R101" s="50">
         <v>176</v>
       </c>
     </row>
-    <row r="102" spans="17:18">
+    <row r="102" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q102" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="R102">
+      <c r="R102" s="50">
         <v>165</v>
       </c>
     </row>
-    <row r="103" spans="17:18">
+    <row r="103" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q103" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="R103">
+      <c r="R103" s="50">
         <v>160</v>
       </c>
     </row>
-    <row r="104" spans="17:18">
+    <row r="104" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q104" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="R104">
+      <c r="R104" s="50">
         <v>138</v>
       </c>
     </row>
-    <row r="105" spans="17:18">
+    <row r="105" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q105" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="R105">
+      <c r="R105" s="50">
         <v>132</v>
       </c>
     </row>
-    <row r="106" spans="17:18">
+    <row r="106" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q106" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="R106">
+      <c r="R106" s="50">
         <v>144</v>
       </c>
     </row>
-    <row r="107" spans="17:18">
+    <row r="107" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q107" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="R107">
+      <c r="R107" s="50">
         <v>155</v>
       </c>
     </row>
-    <row r="108" spans="17:18">
+    <row r="108" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q108" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="R108" s="50">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="109" spans="17:18" x14ac:dyDescent="0.2">
+      <c r="Q109" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="R109" s="50">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="110" spans="17:18" x14ac:dyDescent="0.2">
+      <c r="Q110" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="R108">
-        <v>12542</v>
+      <c r="R110" s="50">
+        <v>12836</v>
       </c>
     </row>
   </sheetData>
@@ -20018,7 +20310,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AA50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="41.1640625" customWidth="1"/>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
@@ -20027,151 +20319,151 @@
     <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="21"/>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="41" t="s">
         <v>133</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="49"/>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="49"/>
-      <c r="U1" s="49"/>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
-      <c r="X1" s="49"/>
-      <c r="Y1" s="49"/>
-      <c r="Z1" s="49"/>
-      <c r="AA1" s="49"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
+      <c r="AA1" s="42"/>
     </row>
-    <row r="2" spans="1:27">
-      <c r="A2" s="45" t="s">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A2" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="43" t="s">
         <v>134</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="41" t="s">
+      <c r="C2" s="44"/>
+      <c r="D2" s="43" t="s">
         <v>135</v>
       </c>
-      <c r="E2" s="42"/>
-      <c r="F2" s="41" t="s">
+      <c r="E2" s="44"/>
+      <c r="F2" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="41" t="s">
+      <c r="G2" s="44"/>
+      <c r="H2" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="I2" s="42"/>
-      <c r="J2" s="41" t="s">
+      <c r="I2" s="44"/>
+      <c r="J2" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="K2" s="42"/>
-      <c r="L2" s="41" t="s">
+      <c r="K2" s="44"/>
+      <c r="L2" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="M2" s="42"/>
-      <c r="N2" s="41" t="s">
+      <c r="M2" s="44"/>
+      <c r="N2" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="O2" s="42"/>
-      <c r="P2" s="41" t="s">
+      <c r="O2" s="44"/>
+      <c r="P2" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="Q2" s="42"/>
-      <c r="R2" s="41" t="s">
+      <c r="Q2" s="44"/>
+      <c r="R2" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="S2" s="42"/>
-      <c r="T2" s="41" t="s">
+      <c r="S2" s="44"/>
+      <c r="T2" s="43" t="s">
         <v>143</v>
       </c>
-      <c r="U2" s="42"/>
-      <c r="V2" s="41" t="s">
+      <c r="U2" s="44"/>
+      <c r="V2" s="43" t="s">
         <v>144</v>
       </c>
-      <c r="W2" s="42"/>
-      <c r="X2" s="41" t="s">
+      <c r="W2" s="44"/>
+      <c r="X2" s="43" t="s">
         <v>145</v>
       </c>
-      <c r="Y2" s="42"/>
-      <c r="Z2" s="41" t="s">
+      <c r="Y2" s="44"/>
+      <c r="Z2" s="43" t="s">
         <v>146</v>
       </c>
-      <c r="AA2" s="42"/>
+      <c r="AA2" s="44"/>
     </row>
-    <row r="3" spans="1:27">
-      <c r="A3" s="46"/>
-      <c r="B3" s="41" t="s">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A3" s="48"/>
+      <c r="B3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="41" t="s">
+      <c r="C3" s="44"/>
+      <c r="D3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="E3" s="42"/>
-      <c r="F3" s="41" t="s">
+      <c r="E3" s="44"/>
+      <c r="F3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="G3" s="42"/>
-      <c r="H3" s="41" t="s">
+      <c r="G3" s="44"/>
+      <c r="H3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="I3" s="42"/>
-      <c r="J3" s="41" t="s">
+      <c r="I3" s="44"/>
+      <c r="J3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="K3" s="42"/>
-      <c r="L3" s="41" t="s">
+      <c r="K3" s="44"/>
+      <c r="L3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="M3" s="42"/>
-      <c r="N3" s="41" t="s">
+      <c r="M3" s="44"/>
+      <c r="N3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="O3" s="42"/>
-      <c r="P3" s="41" t="s">
+      <c r="O3" s="44"/>
+      <c r="P3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="Q3" s="42"/>
-      <c r="R3" s="41" t="s">
+      <c r="Q3" s="44"/>
+      <c r="R3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="S3" s="42"/>
-      <c r="T3" s="41" t="s">
+      <c r="S3" s="44"/>
+      <c r="T3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="U3" s="42"/>
-      <c r="V3" s="41" t="s">
+      <c r="U3" s="44"/>
+      <c r="V3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="W3" s="42"/>
-      <c r="X3" s="41" t="s">
+      <c r="W3" s="44"/>
+      <c r="X3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="Y3" s="42"/>
-      <c r="Z3" s="41" t="s">
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="43" t="s">
         <v>147</v>
       </c>
-      <c r="AA3" s="42"/>
+      <c r="AA3" s="44"/>
     </row>
-    <row r="4" spans="1:27">
-      <c r="A4" s="47"/>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A4" s="49"/>
       <c r="B4" s="23" t="s">
         <v>148</v>
       </c>
@@ -20251,7 +20543,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>14</v>
       </c>
@@ -20334,7 +20626,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:27">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
         <v>18</v>
       </c>
@@ -20417,7 +20709,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>19</v>
       </c>
@@ -20500,7 +20792,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>15</v>
       </c>
@@ -20583,7 +20875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
@@ -20666,7 +20958,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:27">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
         <v>20</v>
       </c>
@@ -20749,7 +21041,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:27">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>16</v>
       </c>
@@ -20832,7 +21124,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:27">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="s">
         <v>150</v>
       </c>
@@ -20915,8 +21207,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:27">
-      <c r="A15" s="45" t="s">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A15" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="22" t="s">
@@ -20959,21 +21251,21 @@
         <v>146</v>
       </c>
       <c r="O15" s="36"/>
-      <c r="P15" s="43"/>
-      <c r="Q15" s="44"/>
-      <c r="R15" s="43"/>
-      <c r="S15" s="44"/>
-      <c r="T15" s="43"/>
-      <c r="U15" s="44"/>
-      <c r="V15" s="43"/>
-      <c r="W15" s="44"/>
-      <c r="X15" s="43"/>
-      <c r="Y15" s="44"/>
-      <c r="Z15" s="43"/>
-      <c r="AA15" s="44"/>
+      <c r="P15" s="45"/>
+      <c r="Q15" s="46"/>
+      <c r="R15" s="45"/>
+      <c r="S15" s="46"/>
+      <c r="T15" s="45"/>
+      <c r="U15" s="46"/>
+      <c r="V15" s="45"/>
+      <c r="W15" s="46"/>
+      <c r="X15" s="45"/>
+      <c r="Y15" s="46"/>
+      <c r="Z15" s="45"/>
+      <c r="AA15" s="46"/>
     </row>
-    <row r="16" spans="1:27">
-      <c r="A16" s="47"/>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A16" s="49"/>
       <c r="B16" s="23" t="s">
         <v>149</v>
       </c>
@@ -21026,7 +21318,7 @@
       <c r="Z16" s="31"/>
       <c r="AA16" s="32"/>
     </row>
-    <row r="17" spans="1:27">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
         <v>14</v>
       </c>
@@ -21095,7 +21387,7 @@
       <c r="Z17" s="33"/>
       <c r="AA17" s="32"/>
     </row>
-    <row r="18" spans="1:27">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
         <v>18</v>
       </c>
@@ -21164,7 +21456,7 @@
       <c r="Z18" s="33"/>
       <c r="AA18" s="32"/>
     </row>
-    <row r="19" spans="1:27">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A19" s="21" t="s">
         <v>19</v>
       </c>
@@ -21233,7 +21525,7 @@
       <c r="Z19" s="33"/>
       <c r="AA19" s="32"/>
     </row>
-    <row r="20" spans="1:27">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
         <v>15</v>
       </c>
@@ -21302,7 +21594,7 @@
       <c r="Z20" s="33"/>
       <c r="AA20" s="32"/>
     </row>
-    <row r="21" spans="1:27">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
@@ -21371,7 +21663,7 @@
       <c r="Z21" s="33"/>
       <c r="AA21" s="32"/>
     </row>
-    <row r="22" spans="1:27">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="21" t="s">
         <v>20</v>
       </c>
@@ -21440,7 +21732,7 @@
       <c r="Z22" s="33"/>
       <c r="AA22" s="32"/>
     </row>
-    <row r="23" spans="1:27">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A23" s="21" t="s">
         <v>16</v>
       </c>
@@ -21509,7 +21801,7 @@
       <c r="Z23" s="33"/>
       <c r="AA23" s="32"/>
     </row>
-    <row r="24" spans="1:27">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A24" s="35"/>
       <c r="N24" s="37"/>
       <c r="P24" s="32"/>
@@ -21525,7 +21817,7 @@
       <c r="Z24" s="32"/>
       <c r="AA24" s="32"/>
     </row>
-    <row r="25" spans="1:27">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
         <v>150</v>
       </c>
@@ -21594,7 +21886,7 @@
       <c r="Z25" s="34"/>
       <c r="AA25" s="32"/>
     </row>
-    <row r="30" spans="1:27">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A30" s="27" t="s">
         <v>151</v>
       </c>
@@ -21638,7 +21930,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:27">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>152</v>
       </c>
@@ -21672,30 +21964,30 @@
       </c>
       <c r="I31" s="1">
         <f>+'Bench Forecast'!I9</f>
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="J31" s="1">
         <f>+'Bench Forecast'!J9</f>
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="K31" s="1">
         <f>+'Bench Forecast'!K9</f>
-        <v>203</v>
+        <v>164</v>
       </c>
       <c r="L31" s="1">
         <f>+'Bench Forecast'!L9</f>
-        <v>215</v>
+        <v>169</v>
       </c>
       <c r="M31" s="1">
         <f>+'Bench Forecast'!M9</f>
-        <v>214</v>
+        <v>172</v>
       </c>
       <c r="N31" s="1">
         <f>+'Bench Forecast'!N9</f>
-        <v>211</v>
+        <v>173</v>
       </c>
     </row>
-    <row r="32" spans="1:27">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>153</v>
       </c>
@@ -21752,7 +22044,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>154</v>
       </c>
@@ -21796,7 +22088,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B36" s="39" t="s">
         <v>155</v>
       </c>
@@ -21804,7 +22096,7 @@
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="38" t="s">
         <v>156</v>
       </c>
@@ -21821,229 +22113,248 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B38" s="50">
+      <c r="B38" s="1">
         <v>170</v>
       </c>
-      <c r="C38" s="50">
+      <c r="C38" s="1">
         <v>159</v>
       </c>
-      <c r="D38" s="50">
+      <c r="D38" s="1">
         <v>159</v>
       </c>
-      <c r="E38" s="50">
+      <c r="E38" s="1">
         <v>488</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B39" s="50">
+      <c r="B39" s="1">
         <v>166</v>
       </c>
-      <c r="C39" s="50">
+      <c r="C39" s="1">
         <v>148</v>
       </c>
-      <c r="D39" s="50">
+      <c r="D39" s="1">
         <v>161</v>
       </c>
-      <c r="E39" s="50">
+      <c r="E39" s="1">
         <v>475</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B40" s="50">
+      <c r="B40" s="1">
         <v>158</v>
       </c>
-      <c r="C40" s="50">
+      <c r="C40" s="1">
         <v>133</v>
       </c>
-      <c r="D40" s="50">
+      <c r="D40" s="1">
         <v>154</v>
       </c>
-      <c r="E40" s="50">
+      <c r="E40" s="1">
         <v>445</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B41" s="50">
+      <c r="B41" s="1">
         <v>138</v>
       </c>
-      <c r="C41" s="50">
+      <c r="C41" s="1">
         <v>138</v>
       </c>
-      <c r="D41" s="50">
+      <c r="D41" s="1">
         <v>156</v>
       </c>
-      <c r="E41" s="50">
+      <c r="E41" s="1">
         <v>432</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B42" s="50">
+      <c r="B42" s="1">
         <v>130</v>
       </c>
-      <c r="C42" s="50">
+      <c r="C42" s="1">
         <v>121</v>
       </c>
-      <c r="D42" s="50">
+      <c r="D42" s="1">
         <v>152</v>
       </c>
-      <c r="E42" s="50">
+      <c r="E42" s="1">
         <v>403</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B43" s="50">
+      <c r="B43" s="1">
         <v>147</v>
       </c>
-      <c r="C43" s="50">
+      <c r="C43" s="1">
         <v>136</v>
       </c>
-      <c r="D43" s="50">
+      <c r="D43" s="1">
         <v>165</v>
       </c>
-      <c r="E43" s="50">
+      <c r="E43" s="1">
         <v>448</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B44" s="50">
+      <c r="B44" s="1">
         <v>155</v>
       </c>
-      <c r="C44" s="50">
+      <c r="C44" s="1">
         <v>119</v>
       </c>
-      <c r="D44" s="50">
+      <c r="D44" s="1">
         <v>175</v>
       </c>
-      <c r="E44" s="50">
+      <c r="E44" s="1">
         <v>449</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B45" s="50">
+      <c r="B45" s="1">
         <v>160</v>
       </c>
-      <c r="C45" s="50">
+      <c r="C45" s="1">
         <v>114</v>
       </c>
-      <c r="D45" s="50">
+      <c r="D45" s="1">
         <v>176</v>
       </c>
-      <c r="E45" s="50">
+      <c r="E45" s="1">
         <v>450</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B46" s="50">
+      <c r="B46" s="1">
         <v>161</v>
       </c>
-      <c r="C46" s="50">
+      <c r="C46" s="1">
         <v>104</v>
       </c>
-      <c r="D46" s="50">
+      <c r="D46" s="1">
         <v>171</v>
       </c>
-      <c r="E46" s="50">
+      <c r="E46" s="1">
         <v>436</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B47" s="50">
+      <c r="B47" s="1">
         <v>203</v>
       </c>
-      <c r="C47" s="50">
+      <c r="C47" s="1">
         <v>112</v>
       </c>
-      <c r="D47" s="50">
+      <c r="D47" s="1">
         <v>196</v>
       </c>
-      <c r="E47" s="50">
+      <c r="E47" s="1">
         <v>511</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B48" s="50">
+      <c r="B48" s="1">
         <v>215</v>
       </c>
-      <c r="C48" s="50">
+      <c r="C48" s="1">
         <v>98</v>
       </c>
-      <c r="D48" s="50">
+      <c r="D48" s="1">
         <v>192</v>
       </c>
-      <c r="E48" s="50">
+      <c r="E48" s="1">
         <v>505</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B49" s="50">
+      <c r="B49" s="1">
         <v>214</v>
       </c>
-      <c r="C49" s="50">
+      <c r="C49" s="1">
         <v>95</v>
       </c>
-      <c r="D49" s="50">
+      <c r="D49" s="1">
         <v>191</v>
       </c>
-      <c r="E49" s="50">
+      <c r="E49" s="1">
         <v>500</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="B50" s="50">
+      <c r="B50" s="1">
         <v>211</v>
       </c>
-      <c r="C50" s="50">
+      <c r="C50" s="1">
         <v>89</v>
       </c>
-      <c r="D50" s="50">
+      <c r="D50" s="1">
         <v>187</v>
       </c>
-      <c r="E50" s="50">
+      <c r="E50" s="1">
         <v>487</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="R15:S15"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="V15:W15"/>
+    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="X15:Y15"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="X3:Y3"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="T15:U15"/>
     <mergeCell ref="B1:AA1"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="D3:E3"/>
@@ -22058,27 +22369,8 @@
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V15:W15"/>
-    <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="X15:Y15"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="Z15:AA15"/>
-    <mergeCell ref="X2:Y2"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="L3:M3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="R15:S15"/>
-    <mergeCell ref="A15:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
data: update NA Bench Forecast with actuals through Wk 03
</commit_message>
<xml_diff>
--- a/NA Bench Forecast.xlsx
+++ b/NA Bench Forecast.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jbondcrx/Desktop/BOB!/Bench Forecast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8DF1DC55-BE05-CF4D-A213-F640ABD9F675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D14E6E7-142A-0B43-9843-2E8F58973591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="600" windowWidth="31020" windowHeight="16080" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="3120" windowWidth="27680" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bench Forecast" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="73" r:id="rId8"/>
-    <pivotCache cacheId="89" r:id="rId9"/>
+    <pivotCache cacheId="95" r:id="rId8"/>
+    <pivotCache cacheId="99" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="180">
   <si>
     <t>Center</t>
   </si>
@@ -583,6 +583,12 @@
   </si>
   <si>
     <t>Fcst</t>
+  </si>
+  <si>
+    <t>4Q26 WK02</t>
+  </si>
+  <si>
+    <t>4Q26 WK03</t>
   </si>
 </sst>
 </file>
@@ -702,7 +708,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -784,6 +790,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -904,7 +916,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1018,6 +1030,24 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
       <protection hidden="1"/>
@@ -1030,20 +1060,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-      <protection hidden="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1051,7 +1069,25 @@
     <cellStyle name="Normal 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -1282,43 +1318,43 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>8.9418777943368111E-2</c:v>
+                  <c:v>7.2528564331843015E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.2463984103328364E-2</c:v>
+                  <c:v>5.7128663686040734E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.8489816194734233E-2</c:v>
+                  <c:v>5.1664182811723795E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.8554396423248884E-2</c:v>
+                  <c:v>6.1599602583209144E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.4580228514654739E-2</c:v>
+                  <c:v>5.663189269746647E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>7.3025335320417287E-2</c:v>
+                  <c:v>6.6567312468951811E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>7.6999503229011432E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.9483358171882762E-2</c:v>
+                  <c:v>7.0044709388971685E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7.9980129160457034E-2</c:v>
+                  <c:v>7.1535022354694486E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.10084451068057626</c:v>
+                  <c:v>9.1902632886239441E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.10680576254346746</c:v>
+                  <c:v>9.2896174863387984E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.10630899155489319</c:v>
+                  <c:v>9.3392945851962242E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.10481867858917039</c:v>
+                  <c:v>9.2896174863387984E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1795,74 +1831,13 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46255.600433680556" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{00000000-000A-0000-FFFF-FFFF9B000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46315.33094803241" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="93" xr:uid="{D0168C38-7504-D94F-B652-797AB12573EA}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A30:N33" sheet="Q3 2025"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="Total Bench" numFmtId="0">
-      <sharedItems count="3">
-        <s v="Q3 26 Forecast"/>
-        <s v="Q3 25 bench"/>
-        <s v="Q3 Original Forecast"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Wk 01" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="159" maxValue="170"/>
-    </cacheField>
-    <cacheField name="Wk 02" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="148" maxValue="166"/>
-    </cacheField>
-    <cacheField name="Wk 03" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="133" maxValue="158"/>
-    </cacheField>
-    <cacheField name="Wk 04" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="138" maxValue="156"/>
-    </cacheField>
-    <cacheField name="Wk 05" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="121" maxValue="152"/>
-    </cacheField>
-    <cacheField name="Wk 06" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="136" maxValue="165"/>
-    </cacheField>
-    <cacheField name="Wk 07" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="119" maxValue="175"/>
-    </cacheField>
-    <cacheField name="Wk 08" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="114" maxValue="176"/>
-    </cacheField>
-    <cacheField name="Wk 09" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="171"/>
-    </cacheField>
-    <cacheField name="Wk 10" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="112" maxValue="203"/>
-    </cacheField>
-    <cacheField name="Wk 11" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="215"/>
-    </cacheField>
-    <cacheField name="Wk 12" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="95" maxValue="214"/>
-    </cacheField>
-    <cacheField name="Wk 13" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="211"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46301.418307291664" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="91" xr:uid="{1D96AD8C-156A-144A-9A6C-C904E8F36591}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="N2:O93" sheet="Historic Bench Data"/>
+    <worksheetSource ref="N2:O95" sheet="Historic Bench Data"/>
   </cacheSource>
   <cacheFields count="2">
     <cacheField name="Wk" numFmtId="0">
-      <sharedItems count="98">
+      <sharedItems count="93">
         <s v="1Q WK 01"/>
         <s v="1Q WK 02"/>
         <s v="1Q WK 03"/>
@@ -1954,13 +1929,8 @@
         <s v="3Q26 WK12"/>
         <s v="3Q26 WK13"/>
         <s v="4Q26 WK01"/>
-        <s v="3Q WK08" u="1"/>
-        <s v="3Q WK09" u="1"/>
-        <s v="3Q WK10" u="1"/>
-        <s v="3Q WK11" u="1"/>
-        <s v="3Q WK12" u="1"/>
-        <s v="3Q WK13" u="1"/>
-        <s v="4Q WK01" u="1"/>
+        <s v="4Q26 WK02"/>
+        <s v="4Q26 WK03"/>
       </sharedItems>
     </cacheField>
     <cacheField name="NA CIC" numFmtId="0">
@@ -1975,61 +1945,69 @@
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
-  <r>
-    <x v="0"/>
-    <n v="170"/>
-    <n v="166"/>
-    <n v="158"/>
-    <n v="138"/>
-    <n v="130"/>
-    <n v="147"/>
-    <n v="155"/>
-    <n v="160"/>
-    <n v="161"/>
-    <n v="203"/>
-    <n v="215"/>
-    <n v="214"/>
-    <n v="211"/>
-  </r>
-  <r>
-    <x v="1"/>
-    <n v="159"/>
-    <n v="148"/>
-    <n v="133"/>
-    <n v="138"/>
-    <n v="121"/>
-    <n v="136"/>
-    <n v="119"/>
-    <n v="114"/>
-    <n v="104"/>
-    <n v="112"/>
-    <n v="98"/>
-    <n v="95"/>
-    <n v="89"/>
-  </r>
-  <r>
-    <x v="2"/>
-    <n v="159"/>
-    <n v="161"/>
-    <n v="154"/>
-    <n v="156"/>
-    <n v="152"/>
-    <n v="165"/>
-    <n v="175"/>
-    <n v="176"/>
-    <n v="171"/>
-    <n v="196"/>
-    <n v="192"/>
-    <n v="191"/>
-    <n v="187"/>
-  </r>
-</pivotCacheRecords>
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Jairo Naranjo" refreshedDate="46315.331267824076" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{00000000-000A-0000-FFFF-FFFF9B000000}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A30:N33" sheet="Q3 2025"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="Total Bench" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Q3 26 Forecast"/>
+        <s v="Q3 25 bench"/>
+        <s v="Q3 Original Forecast"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Wk 01" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="90" maxValue="159"/>
+    </cacheField>
+    <cacheField name="Wk 02" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="89" maxValue="161"/>
+    </cacheField>
+    <cacheField name="Wk 03" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="90" maxValue="154"/>
+    </cacheField>
+    <cacheField name="Wk 04" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="104" maxValue="156"/>
+    </cacheField>
+    <cacheField name="Wk 05" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="93" maxValue="152"/>
+    </cacheField>
+    <cacheField name="Wk 06" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="102" maxValue="165"/>
+    </cacheField>
+    <cacheField name="Wk 07" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="101" maxValue="175"/>
+    </cacheField>
+    <cacheField name="Wk 08" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="93" maxValue="176"/>
+    </cacheField>
+    <cacheField name="Wk 09" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="101" maxValue="171"/>
+    </cacheField>
+    <cacheField name="Wk 10" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="113" maxValue="203"/>
+    </cacheField>
+    <cacheField name="Wk 11" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="86" maxValue="215"/>
+    </cacheField>
+    <cacheField name="Wk 12" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="88" maxValue="214"/>
+    </cacheField>
+    <cacheField name="Wk 13" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="98" maxValue="211"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="91">
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="93">
   <r>
     <x v="0"/>
     <n v="268"/>
@@ -2394,15 +2372,76 @@
     <x v="90"/>
     <n v="179"/>
   </r>
+  <r>
+    <x v="91"/>
+    <n v="180"/>
+  </r>
+  <r>
+    <x v="92"/>
+    <n v="104"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="3">
+  <r>
+    <x v="0"/>
+    <n v="146"/>
+    <n v="115"/>
+    <n v="151"/>
+    <n v="132"/>
+    <n v="120"/>
+    <n v="142"/>
+    <n v="155"/>
+    <n v="160"/>
+    <n v="161"/>
+    <n v="203"/>
+    <n v="215"/>
+    <n v="214"/>
+    <n v="211"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="90"/>
+    <n v="89"/>
+    <n v="90"/>
+    <n v="104"/>
+    <n v="93"/>
+    <n v="102"/>
+    <n v="101"/>
+    <n v="93"/>
+    <n v="101"/>
+    <n v="113"/>
+    <n v="86"/>
+    <n v="88"/>
+    <n v="98"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="159"/>
+    <n v="161"/>
+    <n v="154"/>
+    <n v="156"/>
+    <n v="152"/>
+    <n v="165"/>
+    <n v="175"/>
+    <n v="176"/>
+    <n v="171"/>
+    <n v="196"/>
+    <n v="192"/>
+    <n v="191"/>
+    <n v="187"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D96FC4B6-4D53-F94A-B121-15BFB8F815F6}" name="PivotTable12" cacheId="89" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
-  <location ref="Q23:R115" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{98A565C3-3010-8D41-86BC-F04070C98C07}" name="PivotTable12" cacheId="95" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+  <location ref="Q23:R117" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="2">
     <pivotField axis="axisRow" showAll="0">
-      <items count="99">
+      <items count="94">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -2487,13 +2526,6 @@
         <item x="81"/>
         <item x="82"/>
         <item x="83"/>
-        <item m="1" x="91"/>
-        <item m="1" x="92"/>
-        <item m="1" x="93"/>
-        <item m="1" x="94"/>
-        <item m="1" x="95"/>
-        <item m="1" x="96"/>
-        <item m="1" x="97"/>
         <item x="84"/>
         <item x="85"/>
         <item x="86"/>
@@ -2501,6 +2533,8 @@
         <item x="88"/>
         <item x="89"/>
         <item x="90"/>
+        <item x="91"/>
+        <item x="92"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -2509,7 +2543,7 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="92">
+  <rowItems count="94">
     <i>
       <x/>
     </i>
@@ -2763,25 +2797,31 @@
       <x v="83"/>
     </i>
     <i>
+      <x v="84"/>
+    </i>
+    <i>
+      <x v="85"/>
+    </i>
+    <i>
+      <x v="86"/>
+    </i>
+    <i>
+      <x v="87"/>
+    </i>
+    <i>
+      <x v="88"/>
+    </i>
+    <i>
+      <x v="89"/>
+    </i>
+    <i>
+      <x v="90"/>
+    </i>
+    <i>
       <x v="91"/>
     </i>
     <i>
       <x v="92"/>
-    </i>
-    <i>
-      <x v="93"/>
-    </i>
-    <i>
-      <x v="94"/>
-    </i>
-    <i>
-      <x v="95"/>
-    </i>
-    <i>
-      <x v="96"/>
-    </i>
-    <i>
-      <x v="97"/>
     </i>
     <i t="grand">
       <x/>
@@ -2883,7 +2923,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable2" cacheId="73" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="44">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="PivotTable2" cacheId="99" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Week " updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="44">
   <location ref="A36:E50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField axis="axisCol" showAll="0">
@@ -2985,7 +3025,7 @@
     <dataField name="  Wk 13" fld="13" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="5">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="13">
@@ -3006,23 +3046,23 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="10">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="9">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="2">
+    <format dxfId="8">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="7">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="6">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -4394,13 +4434,13 @@
         <v>14</v>
       </c>
       <c r="B2" s="12">
-        <v>56</v>
-      </c>
-      <c r="C2" s="8">
-        <v>64</v>
-      </c>
-      <c r="D2" s="8">
-        <v>56</v>
+        <v>51</v>
+      </c>
+      <c r="C2" s="42">
+        <v>39</v>
+      </c>
+      <c r="D2" s="42">
+        <v>43</v>
       </c>
       <c r="E2" s="8">
         <v>46</v>
@@ -4438,16 +4478,16 @@
         <v>15</v>
       </c>
       <c r="B3" s="12">
-        <v>6</v>
-      </c>
-      <c r="C3" s="11">
-        <v>2</v>
-      </c>
-      <c r="D3" s="11">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="C3" s="42">
+        <v>7</v>
+      </c>
+      <c r="D3" s="42">
+        <v>5</v>
       </c>
       <c r="E3" s="11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F3" s="11">
         <v>3</v>
@@ -4482,12 +4522,12 @@
         <v>16</v>
       </c>
       <c r="B4" s="12">
-        <v>26</v>
-      </c>
-      <c r="C4" s="8">
-        <v>19</v>
-      </c>
-      <c r="D4" s="8">
+        <v>27</v>
+      </c>
+      <c r="C4" s="42">
+        <v>23</v>
+      </c>
+      <c r="D4" s="42">
         <v>19</v>
       </c>
       <c r="E4" s="8">
@@ -4526,43 +4566,43 @@
         <v>17</v>
       </c>
       <c r="B5" s="12">
-        <v>31</v>
-      </c>
-      <c r="C5" s="11">
-        <v>32</v>
-      </c>
-      <c r="D5" s="11">
-        <v>31</v>
+        <v>24</v>
+      </c>
+      <c r="C5" s="42">
+        <v>15</v>
+      </c>
+      <c r="D5" s="42">
+        <v>10</v>
       </c>
       <c r="E5" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="F5" s="11">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G5" s="11">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H5" s="11">
         <v>23</v>
       </c>
       <c r="I5" s="11">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="J5" s="11">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="K5" s="11">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="L5" s="11">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="M5" s="11">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="N5" s="11">
-        <v>64</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -4570,12 +4610,12 @@
         <v>18</v>
       </c>
       <c r="B6" s="12">
-        <v>15</v>
-      </c>
-      <c r="C6" s="8">
-        <v>15</v>
-      </c>
-      <c r="D6" s="8">
+        <v>14</v>
+      </c>
+      <c r="C6" s="42">
+        <v>11</v>
+      </c>
+      <c r="D6" s="42">
         <v>14</v>
       </c>
       <c r="E6" s="8">
@@ -4616,11 +4656,11 @@
       <c r="B7" s="12">
         <v>12</v>
       </c>
-      <c r="C7" s="11">
-        <v>12</v>
-      </c>
-      <c r="D7" s="11">
-        <v>12</v>
+      <c r="C7" s="42">
+        <v>9</v>
+      </c>
+      <c r="D7" s="42">
+        <v>4</v>
       </c>
       <c r="E7" s="11">
         <v>10</v>
@@ -4658,22 +4698,22 @@
         <v>20</v>
       </c>
       <c r="B8" s="12">
-        <v>34</v>
-      </c>
-      <c r="C8" s="8">
-        <v>22</v>
-      </c>
-      <c r="D8" s="8">
-        <v>24</v>
+        <v>13</v>
+      </c>
+      <c r="C8" s="42">
+        <v>11</v>
+      </c>
+      <c r="D8" s="42">
+        <v>9</v>
       </c>
       <c r="E8" s="8">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F8" s="8">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G8" s="8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H8" s="8">
         <v>19</v>
@@ -4703,27 +4743,27 @@
       </c>
       <c r="B9" s="6">
         <f t="shared" ref="B9:N9" si="0">SUM(B2:B8)</f>
-        <v>180</v>
+        <v>146</v>
       </c>
       <c r="C9" s="6">
         <f t="shared" si="0"/>
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="D9" s="6">
         <f t="shared" si="0"/>
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="E9" s="6">
         <f t="shared" si="0"/>
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="F9" s="6">
         <f t="shared" si="0"/>
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="G9" s="6">
         <f t="shared" si="0"/>
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="H9" s="6">
         <f t="shared" si="0"/>
@@ -4731,27 +4771,27 @@
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="J9" s="6">
         <f t="shared" si="0"/>
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="K9" s="6">
         <f t="shared" si="0"/>
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="L9" s="6">
         <f t="shared" si="0"/>
-        <v>215</v>
+        <v>187</v>
       </c>
       <c r="M9" s="6">
         <f t="shared" si="0"/>
-        <v>214</v>
+        <v>188</v>
       </c>
       <c r="N9" s="6">
         <f t="shared" si="0"/>
-        <v>211</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -4760,27 +4800,27 @@
       </c>
       <c r="B10" s="7">
         <f t="shared" ref="B10:N10" si="1">+B9/$B$11</f>
-        <v>8.9418777943368111E-2</v>
+        <v>7.2528564331843015E-2</v>
       </c>
       <c r="C10" s="7">
         <f t="shared" si="1"/>
-        <v>8.2463984103328364E-2</v>
+        <v>5.7128663686040734E-2</v>
       </c>
       <c r="D10" s="7">
         <f t="shared" si="1"/>
-        <v>7.8489816194734233E-2</v>
+        <v>5.1664182811723795E-2</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="1"/>
-        <v>6.8554396423248884E-2</v>
+        <v>6.1599602583209144E-2</v>
       </c>
       <c r="F10" s="7">
         <f t="shared" si="1"/>
-        <v>6.4580228514654739E-2</v>
+        <v>5.663189269746647E-2</v>
       </c>
       <c r="G10" s="7">
         <f t="shared" si="1"/>
-        <v>7.3025335320417287E-2</v>
+        <v>6.6567312468951811E-2</v>
       </c>
       <c r="H10" s="7">
         <f t="shared" si="1"/>
@@ -4788,27 +4828,27 @@
       </c>
       <c r="I10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9483358171882762E-2</v>
+        <v>7.0044709388971685E-2</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="1"/>
-        <v>7.9980129160457034E-2</v>
+        <v>7.1535022354694486E-2</v>
       </c>
       <c r="K10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10084451068057626</v>
+        <v>9.1902632886239441E-2</v>
       </c>
       <c r="L10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10680576254346746</v>
+        <v>9.2896174863387984E-2</v>
       </c>
       <c r="M10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10630899155489319</v>
+        <v>9.3392945851962242E-2</v>
       </c>
       <c r="N10" s="7">
         <f t="shared" si="1"/>
-        <v>0.10481867858917039</v>
+        <v>9.2896174863387984E-2</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -4821,20 +4861,13 @@
       <c r="C11" s="10"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="N16">
-        <v>136</v>
-      </c>
+      <c r="N16"/>
     </row>
     <row r="17" spans="14:14" x14ac:dyDescent="0.2">
-      <c r="N17">
-        <v>180</v>
-      </c>
+      <c r="N17"/>
     </row>
     <row r="18" spans="14:14" x14ac:dyDescent="0.2">
-      <c r="N18">
-        <f>+N17-N16</f>
-        <v>44</v>
-      </c>
+      <c r="N18"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -4845,7 +4878,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:R115"/>
+  <dimension ref="A1:R117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -5966,7 +5999,7 @@
       <c r="Q24" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="R24" s="45">
+      <c r="R24" s="50">
         <v>268</v>
       </c>
     </row>
@@ -6018,7 +6051,7 @@
       <c r="Q25" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="R25" s="45">
+      <c r="R25" s="50">
         <v>290</v>
       </c>
     </row>
@@ -6070,7 +6103,7 @@
       <c r="Q26" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="R26" s="45">
+      <c r="R26" s="50">
         <v>227</v>
       </c>
     </row>
@@ -6122,7 +6155,7 @@
       <c r="Q27" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="R27" s="45">
+      <c r="R27" s="50">
         <v>228</v>
       </c>
     </row>
@@ -6174,7 +6207,7 @@
       <c r="Q28" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="R28" s="45">
+      <c r="R28" s="50">
         <v>214</v>
       </c>
     </row>
@@ -6226,7 +6259,7 @@
       <c r="Q29" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="R29" s="45">
+      <c r="R29" s="50">
         <v>225</v>
       </c>
     </row>
@@ -6278,7 +6311,7 @@
       <c r="Q30" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="R30" s="45">
+      <c r="R30" s="50">
         <v>207</v>
       </c>
     </row>
@@ -6330,7 +6363,7 @@
       <c r="Q31" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="R31" s="45">
+      <c r="R31" s="50">
         <v>200</v>
       </c>
     </row>
@@ -6382,7 +6415,7 @@
       <c r="Q32" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="R32" s="45">
+      <c r="R32" s="50">
         <v>189</v>
       </c>
     </row>
@@ -6433,7 +6466,7 @@
       <c r="Q33" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="R33" s="45">
+      <c r="R33" s="50">
         <v>180</v>
       </c>
     </row>
@@ -6484,7 +6517,7 @@
       <c r="Q34" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="R34" s="45">
+      <c r="R34" s="50">
         <v>167</v>
       </c>
     </row>
@@ -6536,7 +6569,7 @@
       <c r="Q35" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="R35" s="45">
+      <c r="R35" s="50">
         <v>154</v>
       </c>
     </row>
@@ -6587,7 +6620,7 @@
       <c r="Q36" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="R36" s="45">
+      <c r="R36" s="50">
         <v>148</v>
       </c>
     </row>
@@ -6638,7 +6671,7 @@
       <c r="Q37" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="R37" s="45">
+      <c r="R37" s="50">
         <v>169</v>
       </c>
     </row>
@@ -6689,7 +6722,7 @@
       <c r="Q38" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="R38" s="45">
+      <c r="R38" s="50">
         <v>142</v>
       </c>
     </row>
@@ -6740,7 +6773,7 @@
       <c r="Q39" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="R39" s="45">
+      <c r="R39" s="50">
         <v>169</v>
       </c>
     </row>
@@ -6791,7 +6824,7 @@
       <c r="Q40" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="R40" s="45">
+      <c r="R40" s="50">
         <v>155</v>
       </c>
     </row>
@@ -6843,7 +6876,7 @@
       <c r="Q41" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="R41" s="45">
+      <c r="R41" s="50">
         <v>164</v>
       </c>
     </row>
@@ -6895,7 +6928,7 @@
       <c r="Q42" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="R42" s="45">
+      <c r="R42" s="50">
         <v>136</v>
       </c>
     </row>
@@ -6947,7 +6980,7 @@
       <c r="Q43" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="R43" s="45">
+      <c r="R43" s="50">
         <v>147</v>
       </c>
     </row>
@@ -6999,7 +7032,7 @@
       <c r="Q44" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="R44" s="45">
+      <c r="R44" s="50">
         <v>146</v>
       </c>
     </row>
@@ -7051,7 +7084,7 @@
       <c r="Q45" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="R45" s="45">
+      <c r="R45" s="50">
         <v>148</v>
       </c>
     </row>
@@ -7103,7 +7136,7 @@
       <c r="Q46" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="R46" s="45">
+      <c r="R46" s="50">
         <v>161</v>
       </c>
     </row>
@@ -7155,7 +7188,7 @@
       <c r="Q47" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="R47" s="45">
+      <c r="R47" s="50">
         <v>159</v>
       </c>
     </row>
@@ -7207,7 +7240,7 @@
       <c r="Q48" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="R48" s="45">
+      <c r="R48" s="50">
         <v>133</v>
       </c>
     </row>
@@ -7259,7 +7292,7 @@
       <c r="Q49" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="R49" s="45">
+      <c r="R49" s="50">
         <v>148</v>
       </c>
     </row>
@@ -7311,7 +7344,7 @@
       <c r="Q50" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="R50" s="45">
+      <c r="R50" s="50">
         <v>181</v>
       </c>
     </row>
@@ -7363,7 +7396,7 @@
       <c r="Q51" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="R51" s="45">
+      <c r="R51" s="50">
         <v>177</v>
       </c>
     </row>
@@ -7415,7 +7448,7 @@
       <c r="Q52" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="R52" s="45">
+      <c r="R52" s="50">
         <v>165</v>
       </c>
     </row>
@@ -7467,7 +7500,7 @@
       <c r="Q53" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="R53" s="45">
+      <c r="R53" s="50">
         <v>168</v>
       </c>
     </row>
@@ -7519,7 +7552,7 @@
       <c r="Q54" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="R54" s="45">
+      <c r="R54" s="50">
         <v>146</v>
       </c>
     </row>
@@ -7571,7 +7604,7 @@
       <c r="Q55" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="R55" s="45">
+      <c r="R55" s="50">
         <v>156</v>
       </c>
     </row>
@@ -7623,7 +7656,7 @@
       <c r="Q56" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="R56" s="45">
+      <c r="R56" s="50">
         <v>158</v>
       </c>
     </row>
@@ -7675,7 +7708,7 @@
       <c r="Q57" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="R57" s="45">
+      <c r="R57" s="50">
         <v>143</v>
       </c>
     </row>
@@ -7727,7 +7760,7 @@
       <c r="Q58" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="R58" s="45">
+      <c r="R58" s="50">
         <v>128</v>
       </c>
     </row>
@@ -7779,7 +7812,7 @@
       <c r="Q59" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="R59" s="45">
+      <c r="R59" s="50">
         <v>134</v>
       </c>
     </row>
@@ -7831,7 +7864,7 @@
       <c r="Q60" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="R60" s="45">
+      <c r="R60" s="50">
         <v>123</v>
       </c>
     </row>
@@ -7883,7 +7916,7 @@
       <c r="Q61" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="R61" s="45">
+      <c r="R61" s="50">
         <v>123</v>
       </c>
     </row>
@@ -7935,7 +7968,7 @@
       <c r="Q62" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="R62" s="45">
+      <c r="R62" s="50">
         <v>112</v>
       </c>
     </row>
@@ -7987,7 +8020,7 @@
       <c r="Q63" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="R63" s="45">
+      <c r="R63" s="50">
         <v>119</v>
       </c>
     </row>
@@ -8039,7 +8072,7 @@
       <c r="Q64" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="R64" s="45">
+      <c r="R64" s="50">
         <v>107</v>
       </c>
     </row>
@@ -8091,7 +8124,7 @@
       <c r="Q65" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="R65" s="45">
+      <c r="R65" s="50">
         <v>110</v>
       </c>
     </row>
@@ -8130,7 +8163,7 @@
         <v>121</v>
       </c>
       <c r="L66" t="str">
-        <f t="shared" ref="L66:L93" si="4">+B66&amp;" "&amp;C66</f>
+        <f t="shared" ref="L66:L94" si="4">+B66&amp;" "&amp;C66</f>
         <v>2Q WK 01</v>
       </c>
       <c r="N66" t="s">
@@ -8142,7 +8175,7 @@
       <c r="Q66" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="R66" s="45">
+      <c r="R66" s="50">
         <v>137</v>
       </c>
     </row>
@@ -8193,7 +8226,7 @@
       <c r="Q67" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="R67" s="45">
+      <c r="R67" s="50">
         <v>124</v>
       </c>
     </row>
@@ -8244,7 +8277,7 @@
       <c r="Q68" s="17" t="s">
         <v>93</v>
       </c>
-      <c r="R68" s="45">
+      <c r="R68" s="50">
         <v>127</v>
       </c>
     </row>
@@ -8295,7 +8328,7 @@
       <c r="Q69" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="R69" s="45">
+      <c r="R69" s="50">
         <v>101</v>
       </c>
     </row>
@@ -8347,7 +8380,7 @@
       <c r="Q70" s="17" t="s">
         <v>95</v>
       </c>
-      <c r="R70" s="45">
+      <c r="R70" s="50">
         <v>116</v>
       </c>
     </row>
@@ -8406,7 +8439,7 @@
       <c r="Q71" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="R71" s="45">
+      <c r="R71" s="50">
         <v>124</v>
       </c>
     </row>
@@ -8458,7 +8491,7 @@
       <c r="Q72" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="R72" s="45">
+      <c r="R72" s="50">
         <v>134</v>
       </c>
     </row>
@@ -8517,7 +8550,7 @@
       <c r="Q73" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="R73" s="45">
+      <c r="R73" s="50">
         <v>113</v>
       </c>
     </row>
@@ -8569,7 +8602,7 @@
       <c r="Q74" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="R74" s="45">
+      <c r="R74" s="50">
         <v>118</v>
       </c>
     </row>
@@ -8628,7 +8661,7 @@
       <c r="Q75" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="R75" s="45">
+      <c r="R75" s="50">
         <v>127</v>
       </c>
     </row>
@@ -8680,7 +8713,7 @@
       <c r="Q76" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="R76" s="45">
+      <c r="R76" s="50">
         <v>231</v>
       </c>
     </row>
@@ -8739,7 +8772,7 @@
       <c r="Q77" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="R77" s="45">
+      <c r="R77" s="50">
         <v>201</v>
       </c>
     </row>
@@ -8790,7 +8823,7 @@
       <c r="Q78" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="R78" s="45">
+      <c r="R78" s="50">
         <v>180</v>
       </c>
     </row>
@@ -8826,7 +8859,7 @@
         <v>18</v>
       </c>
       <c r="K79" s="15">
-        <f t="shared" ref="K79:K93" si="6">SUM(D79:J79)</f>
+        <f t="shared" ref="K79:K92" si="6">SUM(D79:J79)</f>
         <v>176</v>
       </c>
       <c r="L79" t="str">
@@ -8842,7 +8875,7 @@
       <c r="Q79" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="R79" s="45">
+      <c r="R79" s="50">
         <v>171</v>
       </c>
     </row>
@@ -8894,7 +8927,7 @@
       <c r="Q80" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="R80" s="45">
+      <c r="R80" s="50">
         <v>148</v>
       </c>
     </row>
@@ -8946,7 +8979,7 @@
       <c r="Q81" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="R81" s="45">
+      <c r="R81" s="50">
         <v>143</v>
       </c>
     </row>
@@ -8998,7 +9031,7 @@
       <c r="Q82" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="R82" s="45">
+      <c r="R82" s="50">
         <v>114</v>
       </c>
     </row>
@@ -9050,7 +9083,7 @@
       <c r="Q83" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="R83" s="45">
+      <c r="R83" s="50">
         <v>110</v>
       </c>
     </row>
@@ -9102,7 +9135,7 @@
       <c r="Q84" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="R84" s="45">
+      <c r="R84" s="50">
         <v>97</v>
       </c>
     </row>
@@ -9154,7 +9187,7 @@
       <c r="Q85" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="R85" s="45">
+      <c r="R85" s="50">
         <v>101</v>
       </c>
     </row>
@@ -9206,7 +9239,7 @@
       <c r="Q86" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="R86" s="45">
+      <c r="R86" s="50">
         <v>78</v>
       </c>
     </row>
@@ -9258,7 +9291,7 @@
       <c r="Q87" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="R87" s="45">
+      <c r="R87" s="50">
         <v>73</v>
       </c>
     </row>
@@ -9310,7 +9343,7 @@
       <c r="Q88" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="R88" s="45">
+      <c r="R88" s="50">
         <v>121</v>
       </c>
     </row>
@@ -9362,7 +9395,7 @@
       <c r="Q89" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="R89" s="45">
+      <c r="R89" s="50">
         <v>117</v>
       </c>
     </row>
@@ -9414,7 +9447,7 @@
       <c r="Q90" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="R90" s="45">
+      <c r="R90" s="50">
         <v>114</v>
       </c>
     </row>
@@ -9466,7 +9499,7 @@
       <c r="Q91" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="R91" s="45">
+      <c r="R91" s="50">
         <v>114</v>
       </c>
     </row>
@@ -9518,11 +9551,11 @@
       <c r="Q92" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="R92" s="45">
+      <c r="R92" s="50">
         <v>114</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="14">
         <v>2026</v>
       </c>
@@ -9569,23 +9602,72 @@
       <c r="Q93" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="R93" s="45">
+      <c r="R93" s="50">
         <v>137</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:18" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="20">
+        <v>2026</v>
+      </c>
+      <c r="B94" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="C94" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D94" s="19">
+        <v>43</v>
+      </c>
+      <c r="E94" s="19">
+        <v>14</v>
+      </c>
+      <c r="F94" s="19">
+        <v>4</v>
+      </c>
+      <c r="G94" s="19">
+        <v>5</v>
+      </c>
+      <c r="H94" s="19">
+        <v>10</v>
+      </c>
+      <c r="I94" s="19">
+        <v>9</v>
+      </c>
+      <c r="J94" s="19">
+        <v>19</v>
+      </c>
+      <c r="K94" s="19">
+        <v>104</v>
+      </c>
+      <c r="L94" t="str">
+        <f t="shared" si="4"/>
+        <v>4Q WK 03</v>
+      </c>
+      <c r="N94" t="s">
+        <v>178</v>
+      </c>
+      <c r="O94" s="15">
+        <v>180</v>
+      </c>
       <c r="Q94" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="R94" s="45">
+      <c r="R94" s="50">
         <v>126</v>
       </c>
     </row>
     <row r="95" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="N95" t="s">
+        <v>179</v>
+      </c>
+      <c r="O95" s="19">
+        <v>104</v>
+      </c>
       <c r="Q95" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="R95" s="45">
+      <c r="R95" s="50">
         <v>151</v>
       </c>
     </row>
@@ -9593,7 +9675,7 @@
       <c r="Q96" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="R96" s="45">
+      <c r="R96" s="50">
         <v>125</v>
       </c>
     </row>
@@ -9601,7 +9683,7 @@
       <c r="Q97" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="R97" s="45">
+      <c r="R97" s="50">
         <v>116</v>
       </c>
     </row>
@@ -9609,7 +9691,7 @@
       <c r="Q98" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="R98" s="45">
+      <c r="R98" s="50">
         <v>145</v>
       </c>
     </row>
@@ -9617,7 +9699,7 @@
       <c r="Q99" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="R99" s="45">
+      <c r="R99" s="50">
         <v>148</v>
       </c>
     </row>
@@ -9625,7 +9707,7 @@
       <c r="Q100" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="R100" s="45">
+      <c r="R100" s="50">
         <v>152</v>
       </c>
     </row>
@@ -9633,7 +9715,7 @@
       <c r="Q101" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="R101" s="45">
+      <c r="R101" s="50">
         <v>176</v>
       </c>
     </row>
@@ -9641,7 +9723,7 @@
       <c r="Q102" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="R102" s="45">
+      <c r="R102" s="50">
         <v>165</v>
       </c>
     </row>
@@ -9649,7 +9731,7 @@
       <c r="Q103" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="R103" s="45">
+      <c r="R103" s="50">
         <v>160</v>
       </c>
     </row>
@@ -9657,7 +9739,7 @@
       <c r="Q104" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="R104" s="45">
+      <c r="R104" s="50">
         <v>138</v>
       </c>
     </row>
@@ -9665,7 +9747,7 @@
       <c r="Q105" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="R105" s="45">
+      <c r="R105" s="50">
         <v>132</v>
       </c>
     </row>
@@ -9673,7 +9755,7 @@
       <c r="Q106" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="R106" s="45">
+      <c r="R106" s="50">
         <v>144</v>
       </c>
     </row>
@@ -9681,7 +9763,7 @@
       <c r="Q107" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="R107" s="45">
+      <c r="R107" s="50">
         <v>155</v>
       </c>
     </row>
@@ -9689,7 +9771,7 @@
       <c r="Q108" s="17" t="s">
         <v>168</v>
       </c>
-      <c r="R108" s="45">
+      <c r="R108" s="50">
         <v>149</v>
       </c>
     </row>
@@ -9697,7 +9779,7 @@
       <c r="Q109" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="R109" s="45">
+      <c r="R109" s="50">
         <v>145</v>
       </c>
     </row>
@@ -9705,7 +9787,7 @@
       <c r="Q110" s="17" t="s">
         <v>170</v>
       </c>
-      <c r="R110" s="45">
+      <c r="R110" s="50">
         <v>158</v>
       </c>
     </row>
@@ -9713,7 +9795,7 @@
       <c r="Q111" s="17" t="s">
         <v>171</v>
       </c>
-      <c r="R111" s="45">
+      <c r="R111" s="50">
         <v>167</v>
       </c>
     </row>
@@ -9721,7 +9803,7 @@
       <c r="Q112" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="R112" s="45">
+      <c r="R112" s="50">
         <v>169</v>
       </c>
     </row>
@@ -9729,7 +9811,7 @@
       <c r="Q113" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="R113" s="45">
+      <c r="R113" s="50">
         <v>169</v>
       </c>
     </row>
@@ -9737,20 +9819,37 @@
       <c r="Q114" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="R114" s="45">
+      <c r="R114" s="50">
         <v>179</v>
       </c>
     </row>
     <row r="115" spans="17:18" x14ac:dyDescent="0.2">
       <c r="Q115" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="R115" s="50">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="116" spans="17:18" x14ac:dyDescent="0.2">
+      <c r="Q116" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="R116" s="50">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="117" spans="17:18" x14ac:dyDescent="0.2">
+      <c r="Q117" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="R115" s="45">
-        <v>13678</v>
+      <c r="R117" s="50">
+        <v>13962</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K32" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -9760,234 +9859,234 @@
   <dimension ref="A1:AA50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="21"/>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="43" t="s">
         <v>175</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="M1" s="46"/>
-      <c r="N1" s="46"/>
-      <c r="O1" s="46"/>
-      <c r="P1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="46"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="46"/>
-      <c r="V1" s="46"/>
-      <c r="W1" s="46"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="46"/>
-      <c r="Z1" s="46"/>
-      <c r="AA1" s="46"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="43"/>
+      <c r="V1" s="43"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="C2" s="48"/>
-      <c r="D2" s="47" t="s">
+      <c r="C2" s="45"/>
+      <c r="D2" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="E2" s="48"/>
-      <c r="F2" s="47" t="s">
+      <c r="E2" s="45"/>
+      <c r="F2" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="G2" s="48"/>
-      <c r="H2" s="47" t="s">
+      <c r="G2" s="45"/>
+      <c r="H2" s="44" t="s">
         <v>136</v>
       </c>
-      <c r="I2" s="48"/>
-      <c r="J2" s="47" t="s">
+      <c r="I2" s="45"/>
+      <c r="J2" s="44" t="s">
         <v>137</v>
       </c>
-      <c r="K2" s="48"/>
-      <c r="L2" s="47" t="s">
+      <c r="K2" s="45"/>
+      <c r="L2" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="M2" s="48"/>
-      <c r="N2" s="47" t="s">
+      <c r="M2" s="45"/>
+      <c r="N2" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="O2" s="48"/>
-      <c r="P2" s="47" t="s">
+      <c r="O2" s="45"/>
+      <c r="P2" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="47" t="s">
+      <c r="Q2" s="45"/>
+      <c r="R2" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="S2" s="48"/>
-      <c r="T2" s="47" t="s">
+      <c r="S2" s="45"/>
+      <c r="T2" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="U2" s="48"/>
-      <c r="V2" s="47" t="s">
+      <c r="U2" s="45"/>
+      <c r="V2" s="44" t="s">
         <v>143</v>
       </c>
-      <c r="W2" s="48"/>
-      <c r="X2" s="47" t="s">
+      <c r="W2" s="45"/>
+      <c r="X2" s="44" t="s">
         <v>144</v>
       </c>
-      <c r="Y2" s="48"/>
-      <c r="Z2" s="47" t="s">
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="44" t="s">
         <v>145</v>
       </c>
-      <c r="AA2" s="48"/>
+      <c r="AA2" s="45"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A3" s="46"/>
-      <c r="B3" s="47" t="s">
+      <c r="A3" s="43"/>
+      <c r="B3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="C3" s="48"/>
-      <c r="D3" s="47" t="s">
+      <c r="C3" s="45"/>
+      <c r="D3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="47" t="s">
+      <c r="E3" s="45"/>
+      <c r="F3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="G3" s="48"/>
-      <c r="H3" s="47" t="s">
+      <c r="G3" s="45"/>
+      <c r="H3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="I3" s="48"/>
-      <c r="J3" s="47" t="s">
+      <c r="I3" s="45"/>
+      <c r="J3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="K3" s="48"/>
-      <c r="L3" s="47" t="s">
+      <c r="K3" s="45"/>
+      <c r="L3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="M3" s="48"/>
-      <c r="N3" s="47" t="s">
+      <c r="M3" s="45"/>
+      <c r="N3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="O3" s="48"/>
-      <c r="P3" s="47" t="s">
+      <c r="O3" s="45"/>
+      <c r="P3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="Q3" s="48"/>
-      <c r="R3" s="47" t="s">
+      <c r="Q3" s="45"/>
+      <c r="R3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="S3" s="48"/>
-      <c r="T3" s="47" t="s">
+      <c r="S3" s="45"/>
+      <c r="T3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="U3" s="48"/>
-      <c r="V3" s="47" t="s">
+      <c r="U3" s="45"/>
+      <c r="V3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="W3" s="48"/>
-      <c r="X3" s="47" t="s">
+      <c r="W3" s="45"/>
+      <c r="X3" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="Y3" s="48"/>
-      <c r="Z3" s="47" t="s">
+      <c r="Y3" s="45"/>
+      <c r="Z3" s="44" t="s">
         <v>177</v>
       </c>
-      <c r="AA3" s="48"/>
+      <c r="AA3" s="45"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A4" s="46"/>
-      <c r="B4" s="49" t="s">
+      <c r="A4" s="43"/>
+      <c r="B4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="D4" s="49" t="s">
+      <c r="D4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="E4" s="49" t="s">
+      <c r="E4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="F4" s="49" t="s">
+      <c r="F4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="G4" s="49" t="s">
+      <c r="G4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="H4" s="49" t="s">
+      <c r="H4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="I4" s="49" t="s">
+      <c r="I4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="J4" s="49" t="s">
+      <c r="J4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="K4" s="49" t="s">
+      <c r="K4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="L4" s="49" t="s">
+      <c r="L4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="M4" s="49" t="s">
+      <c r="M4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="N4" s="49" t="s">
+      <c r="N4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="O4" s="49" t="s">
+      <c r="O4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="P4" s="49" t="s">
+      <c r="P4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="Q4" s="49" t="s">
+      <c r="Q4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="R4" s="49" t="s">
+      <c r="R4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="S4" s="49" t="s">
+      <c r="S4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="T4" s="49" t="s">
+      <c r="T4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="U4" s="49" t="s">
+      <c r="U4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="V4" s="49" t="s">
+      <c r="V4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="W4" s="49" t="s">
+      <c r="W4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="X4" s="49" t="s">
+      <c r="X4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="Y4" s="49" t="s">
+      <c r="Y4" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="Z4" s="49" t="s">
+      <c r="Z4" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="AA4" s="49" t="s">
+      <c r="AA4" s="41" t="s">
         <v>147</v>
       </c>
     </row>
@@ -10656,7 +10755,7 @@
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A15" s="43" t="s">
+      <c r="A15" s="48" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="22" t="s">
@@ -10699,21 +10798,21 @@
         <v>145</v>
       </c>
       <c r="O15" s="36"/>
-      <c r="P15" s="41"/>
-      <c r="Q15" s="42"/>
-      <c r="R15" s="41"/>
-      <c r="S15" s="42"/>
-      <c r="T15" s="41"/>
-      <c r="U15" s="42"/>
-      <c r="V15" s="41"/>
-      <c r="W15" s="42"/>
-      <c r="X15" s="41"/>
-      <c r="Y15" s="42"/>
-      <c r="Z15" s="41"/>
-      <c r="AA15" s="42"/>
+      <c r="P15" s="46"/>
+      <c r="Q15" s="47"/>
+      <c r="R15" s="46"/>
+      <c r="S15" s="47"/>
+      <c r="T15" s="46"/>
+      <c r="U15" s="47"/>
+      <c r="V15" s="46"/>
+      <c r="W15" s="47"/>
+      <c r="X15" s="46"/>
+      <c r="Y15" s="47"/>
+      <c r="Z15" s="46"/>
+      <c r="AA15" s="47"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A16" s="44"/>
+      <c r="A16" s="49"/>
       <c r="B16" s="23" t="s">
         <v>147</v>
       </c>
@@ -11384,27 +11483,27 @@
       </c>
       <c r="B31" s="1">
         <f>+'Bench Forecast'!B9</f>
-        <v>180</v>
+        <v>146</v>
       </c>
       <c r="C31" s="1">
         <f>+'Bench Forecast'!C9</f>
-        <v>166</v>
+        <v>115</v>
       </c>
       <c r="D31" s="1">
         <f>+'Bench Forecast'!D9</f>
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="E31" s="1">
         <f>+'Bench Forecast'!E9</f>
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="F31" s="1">
         <f>+'Bench Forecast'!F9</f>
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="G31" s="1">
         <f>+'Bench Forecast'!G9</f>
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="H31" s="1">
         <f>+'Bench Forecast'!H9</f>
@@ -11412,27 +11511,27 @@
       </c>
       <c r="I31" s="1">
         <f>+'Bench Forecast'!I9</f>
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="J31" s="1">
         <f>+'Bench Forecast'!J9</f>
-        <v>161</v>
+        <v>144</v>
       </c>
       <c r="K31" s="1">
         <f>+'Bench Forecast'!K9</f>
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="L31" s="1">
         <f>+'Bench Forecast'!L9</f>
-        <v>215</v>
+        <v>187</v>
       </c>
       <c r="M31" s="1">
         <f>+'Bench Forecast'!M9</f>
-        <v>214</v>
+        <v>188</v>
       </c>
       <c r="N31" s="1">
         <f>+'Bench Forecast'!N9</f>
-        <v>211</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.2">
@@ -11565,221 +11664,221 @@
       <c r="A38" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B38" s="1">
-        <v>170</v>
-      </c>
-      <c r="C38" s="1">
+      <c r="B38" s="51">
+        <v>146</v>
+      </c>
+      <c r="C38" s="51">
+        <v>90</v>
+      </c>
+      <c r="D38" s="51">
         <v>159</v>
       </c>
-      <c r="D38" s="1">
-        <v>159</v>
-      </c>
-      <c r="E38" s="1">
-        <v>488</v>
+      <c r="E38" s="51">
+        <v>395</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B39" s="1">
-        <v>166</v>
-      </c>
-      <c r="C39" s="1">
-        <v>148</v>
-      </c>
-      <c r="D39" s="1">
+      <c r="B39" s="51">
+        <v>115</v>
+      </c>
+      <c r="C39" s="51">
+        <v>89</v>
+      </c>
+      <c r="D39" s="51">
         <v>161</v>
       </c>
-      <c r="E39" s="1">
-        <v>475</v>
+      <c r="E39" s="51">
+        <v>365</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="B40" s="1">
-        <v>158</v>
-      </c>
-      <c r="C40" s="1">
-        <v>133</v>
-      </c>
-      <c r="D40" s="1">
+      <c r="B40" s="51">
+        <v>151</v>
+      </c>
+      <c r="C40" s="51">
+        <v>90</v>
+      </c>
+      <c r="D40" s="51">
         <v>154</v>
       </c>
-      <c r="E40" s="1">
-        <v>445</v>
+      <c r="E40" s="51">
+        <v>395</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B41" s="1">
-        <v>138</v>
-      </c>
-      <c r="C41" s="1">
-        <v>138</v>
-      </c>
-      <c r="D41" s="1">
+      <c r="B41" s="51">
+        <v>132</v>
+      </c>
+      <c r="C41" s="51">
+        <v>104</v>
+      </c>
+      <c r="D41" s="51">
         <v>156</v>
       </c>
-      <c r="E41" s="1">
-        <v>432</v>
+      <c r="E41" s="51">
+        <v>392</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B42" s="1">
-        <v>130</v>
-      </c>
-      <c r="C42" s="1">
-        <v>121</v>
-      </c>
-      <c r="D42" s="1">
+      <c r="B42" s="51">
+        <v>120</v>
+      </c>
+      <c r="C42" s="51">
+        <v>93</v>
+      </c>
+      <c r="D42" s="51">
         <v>152</v>
       </c>
-      <c r="E42" s="1">
-        <v>403</v>
+      <c r="E42" s="51">
+        <v>365</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B43" s="1">
-        <v>147</v>
-      </c>
-      <c r="C43" s="1">
-        <v>136</v>
-      </c>
-      <c r="D43" s="1">
+      <c r="B43" s="51">
+        <v>142</v>
+      </c>
+      <c r="C43" s="51">
+        <v>102</v>
+      </c>
+      <c r="D43" s="51">
         <v>165</v>
       </c>
-      <c r="E43" s="1">
-        <v>448</v>
+      <c r="E43" s="51">
+        <v>409</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="51">
         <v>155</v>
       </c>
-      <c r="C44" s="1">
-        <v>119</v>
-      </c>
-      <c r="D44" s="1">
+      <c r="C44" s="51">
+        <v>101</v>
+      </c>
+      <c r="D44" s="51">
         <v>175</v>
       </c>
-      <c r="E44" s="1">
-        <v>449</v>
+      <c r="E44" s="51">
+        <v>431</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="51">
         <v>160</v>
       </c>
-      <c r="C45" s="1">
-        <v>114</v>
-      </c>
-      <c r="D45" s="1">
+      <c r="C45" s="51">
+        <v>93</v>
+      </c>
+      <c r="D45" s="51">
         <v>176</v>
       </c>
-      <c r="E45" s="1">
-        <v>450</v>
+      <c r="E45" s="51">
+        <v>429</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="51">
         <v>161</v>
       </c>
-      <c r="C46" s="1">
-        <v>104</v>
-      </c>
-      <c r="D46" s="1">
+      <c r="C46" s="51">
+        <v>101</v>
+      </c>
+      <c r="D46" s="51">
         <v>171</v>
       </c>
-      <c r="E46" s="1">
-        <v>436</v>
+      <c r="E46" s="51">
+        <v>433</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="51">
         <v>203</v>
       </c>
-      <c r="C47" s="1">
-        <v>112</v>
-      </c>
-      <c r="D47" s="1">
+      <c r="C47" s="51">
+        <v>113</v>
+      </c>
+      <c r="D47" s="51">
         <v>196</v>
       </c>
-      <c r="E47" s="1">
-        <v>511</v>
+      <c r="E47" s="51">
+        <v>512</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="51">
         <v>215</v>
       </c>
-      <c r="C48" s="1">
-        <v>98</v>
-      </c>
-      <c r="D48" s="1">
+      <c r="C48" s="51">
+        <v>86</v>
+      </c>
+      <c r="D48" s="51">
         <v>192</v>
       </c>
-      <c r="E48" s="1">
-        <v>505</v>
+      <c r="E48" s="51">
+        <v>493</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="51">
         <v>214</v>
       </c>
-      <c r="C49" s="1">
-        <v>95</v>
-      </c>
-      <c r="D49" s="1">
+      <c r="C49" s="51">
+        <v>88</v>
+      </c>
+      <c r="D49" s="51">
         <v>191</v>
       </c>
-      <c r="E49" s="1">
-        <v>500</v>
+      <c r="E49" s="51">
+        <v>493</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="51">
         <v>211</v>
       </c>
-      <c r="C50" s="1">
-        <v>89</v>
-      </c>
-      <c r="D50" s="1">
+      <c r="C50" s="51">
+        <v>98</v>
+      </c>
+      <c r="D50" s="51">
         <v>187</v>
       </c>
-      <c r="E50" s="1">
-        <v>487</v>
+      <c r="E50" s="51">
+        <v>496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>